<commit_message>
docs: add staged burn down controls
</commit_message>
<xml_diff>
--- a/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
+++ b/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
@@ -18,33 +18,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="179">
   <si>
     <t>Amped Up Network Financial Model</t>
   </si>
   <si>
-    <t>Purpose</t>
-  </si>
-  <si>
-    <t>Editable 12-month founder-led launch model. Change yellow cells on the Assumptions sheet; all cash-flow, funding, and run-rate calculations update automatically when opened in Excel, Numbers, or Google Sheets.</t>
-  </si>
-  <si>
-    <t>Model scope</t>
-  </si>
-  <si>
-    <t>This model separates the mature first-market run rate from the launch-year cash ramp. It assumes partner launch fees are collected in the month shown, annual member dues are collected upfront, and no managed-service or expert-work margin is included unless entered in Assumptions.</t>
-  </si>
-  <si>
-    <t>Funding logic</t>
-  </si>
-  <si>
-    <t>The Funding sheet calculates the minimum capital needed to keep the requested reserve intact at the lowest point in the 12-month ramp. It does not recommend debt; compare founder capital, partner/member receipts, a line of credit, or investment using the scenarios on that sheet.</t>
-  </si>
-  <si>
-    <t>Important</t>
-  </si>
-  <si>
-    <t>All figures are planning assumptions, not financial advice, a forecast, or earnings representation. Replace them with actual lease, payroll, vendor, insurance, tax, payment-fee, and partner-contract terms before relying on this model for financing.</t>
+    <t>How to use</t>
+  </si>
+  <si>
+    <t>Edit yellow cells only. Assumptions controls recurring cost and price drivers; yellow rows on 12 Month Cash Flow control launch timing, one-time payment timing, and outside funding/debt/investment draws. Formula rows recalculate automatically when opened in Excel, Numbers, or Google Sheets.</t>
+  </si>
+  <si>
+    <t>Backloading</t>
+  </si>
+  <si>
+    <t>Set each recurring expense start month on Assumptions. Move legal, equipment, and other one-time payments across the yellow schedule on 12 Month Cash Flow. Use the yellow External funding draw row only when a loan, investment, or founder contribution is expected to close; do not count an uncommitted source as cash.</t>
+  </si>
+  <si>
+    <t>Capital decision</t>
+  </si>
+  <si>
+    <t>Funding calculates the reserve requirement from the lowest cash point before funding. It shows the difference between minimum required funding and the timing of a proposed draw. All figures are planning assumptions, not financial advice or an earnings claim.</t>
   </si>
   <si>
     <t>Editable Assumptions</t>
@@ -71,48 +65,69 @@
     <t>Founder-led draw and targeted operating support; excludes replacement-value labor.</t>
   </si>
   <si>
+    <t>Founder / operations start month</t>
+  </si>
+  <si>
+    <t>month number</t>
+  </si>
+  <si>
+    <t>Delay draw until the business reaches the chosen milestone; do not defer necessary safety/compliance work.</t>
+  </si>
+  <si>
     <t>Engineering / product monthly cash cost</t>
   </si>
   <si>
-    <t>Scoped contractors for security, payments, workflows, and integrations.</t>
+    <t>Contract only milestone-critical work.</t>
+  </si>
+  <si>
+    <t>Engineering / product start month</t>
   </si>
   <si>
     <t>Content / social monthly cash cost</t>
   </si>
   <si>
-    <t>Family-assisted production plus targeted outside work; excludes imputed family labor.</t>
+    <t>Family-assisted production plus targeted outside work.</t>
+  </si>
+  <si>
+    <t>Content / social start month</t>
   </si>
   <si>
     <t>Software / payments / data monthly cost</t>
   </si>
   <si>
-    <t>Hosting, communications, analytics, CRM, and payment-related tooling.</t>
+    <t>Hosting, communications, analytics, CRM, and payment tooling.</t>
+  </si>
+  <si>
+    <t>Software / payments / data start month</t>
   </si>
   <si>
     <t>Marketing / event monthly cash cost</t>
   </si>
   <si>
-    <t>Partner-hosted and co-funded activations; avoid large self-funded events.</t>
+    <t>Partner-hosted and co-funded events; no self-funded large shows in year one.</t>
+  </si>
+  <si>
+    <t>Marketing / event start month</t>
   </si>
   <si>
     <t>Premises branding / place-based media monthly cost</t>
   </si>
   <si>
-    <t>Partner kits, QR assets, and small local media tests before billboard-scale spend.</t>
+    <t>Partner kits and small local media tests before billboards.</t>
+  </si>
+  <si>
+    <t>Premises branding / place-based media start month</t>
   </si>
   <si>
     <t>Connected Garage monthly pilot cost</t>
   </si>
   <si>
-    <t>Tesla-first Tessie pilot, secure storage/processing, and support.</t>
+    <t>Tesla-first Tessie pilot, secure telemetry storage/processing, and support.</t>
   </si>
   <si>
     <t>Connected Garage pilot start month</t>
   </si>
   <si>
-    <t>month number</t>
-  </si>
-  <si>
     <t>Set to 13 to defer beyond the first year.</t>
   </si>
   <si>
@@ -122,40 +137,7 @@
     <t>cash balance</t>
   </si>
   <si>
-    <t>Desired minimum cash balance, not an operating expense.</t>
-  </si>
-  <si>
-    <t>Legal / compliance: Month 1</t>
-  </si>
-  <si>
-    <t>one time</t>
-  </si>
-  <si>
-    <t>Program structure, franchise, referral, privacy, contracts, insurance, and terms.</t>
-  </si>
-  <si>
-    <t>Legal / compliance: Month 2</t>
-  </si>
-  <si>
-    <t>Legal / compliance: Month 3</t>
-  </si>
-  <si>
-    <t>Legal / compliance: Month 4</t>
-  </si>
-  <si>
-    <t>Legal / compliance: Month 9</t>
-  </si>
-  <si>
-    <t>Legal / compliance: Month 12</t>
-  </si>
-  <si>
-    <t>Content equipment: Month 2</t>
-  </si>
-  <si>
-    <t>Camera, audio, lighting, editing/storage; rent specialty gear.</t>
-  </si>
-  <si>
-    <t>Content equipment: Month 3</t>
+    <t>Minimum desired cash balance, not an operating expense.</t>
   </si>
   <si>
     <t>Full repair-partner launch fee</t>
@@ -209,13 +191,13 @@
     <t>Vendor-funded or local partner campaign.</t>
   </si>
   <si>
-    <t>Starting founder / investor capital</t>
+    <t>Starting founder capital</t>
   </si>
   <si>
     <t>cash</t>
   </si>
   <si>
-    <t>Initial cash committed before Month 1. Funding sheet calculates the minimum required.</t>
+    <t>Cash already available before Month 1. Keep at zero when modeling a fully backloaded draw.</t>
   </si>
   <si>
     <t>Managed-service contribution margin</t>
@@ -233,7 +215,7 @@
     <t>12-Month Founder-Led Cash Burn-Down</t>
   </si>
   <si>
-    <t>Yellow input rows set the market-launch ramp. Formula rows calculate funding and cash position.</t>
+    <t>Yellow cells are timing or funding inputs. All other monthly values are formulas.</t>
   </si>
   <si>
     <t>Driver / Cash Flow</t>
@@ -296,6 +278,15 @@
     <t>Vendor / local campaigns</t>
   </si>
   <si>
+    <t>Legal / compliance payment schedule</t>
+  </si>
+  <si>
+    <t>Equipment / initial production payment schedule</t>
+  </si>
+  <si>
+    <t>External funding draw: debt / investment / founder</t>
+  </si>
+  <si>
     <t>Revenue</t>
   </si>
   <si>
@@ -356,7 +347,7 @@
     <t>Legal / compliance</t>
   </si>
   <si>
-    <t>Content equipment</t>
+    <t>Equipment / initial production</t>
   </si>
   <si>
     <t>Total operating expenses</t>
@@ -371,7 +362,10 @@
     <t>Cumulative cash before funding</t>
   </si>
   <si>
-    <t>Opening cash after funding</t>
+    <t>Opening cash</t>
+  </si>
+  <si>
+    <t>External funding draw</t>
   </si>
   <si>
     <t>Closing cash</t>
@@ -380,7 +374,7 @@
     <t>Cash above / (below) reserve</t>
   </si>
   <si>
-    <t>Funding Waterfall and Capital Decision</t>
+    <t>Funding Waterfall and Capital Timing</t>
   </si>
   <si>
     <t>Measure</t>
@@ -395,61 +389,61 @@
     <t>Launch-year revenue receipts</t>
   </si>
   <si>
-    <t>Partner launch fees, MRR, annual memberships, booking fees, campaign contributions, and optional product lines.</t>
+    <t>Cash receipts from the launch schedule, recurring memberships, annual dues, booking fees, and campaign contributions.</t>
   </si>
   <si>
     <t>Launch-year operating expenses</t>
   </si>
   <si>
-    <t>Cash costs only; excludes reserve and replacement value of founder/family labor.</t>
+    <t>Cash operating costs, including the editable legal and equipment schedules.</t>
   </si>
   <si>
     <t>Launch-year net operating cash flow</t>
   </si>
   <si>
-    <t>Negative means the market ramp consumes cash before funding.</t>
+    <t>Negative means the ramp consumes cash before founder or external funding.</t>
   </si>
   <si>
     <t>Lowest cumulative cash before funding</t>
   </si>
   <si>
-    <t>Worst cash point if no opening capital is injected.</t>
+    <t>Worst point if no starting capital or external funding is drawn.</t>
   </si>
   <si>
     <t>Required reserve</t>
   </si>
   <si>
-    <t>Minimum desired cash buffer.</t>
+    <t>Minimum desired balance.</t>
   </si>
   <si>
     <t>Minimum funding to preserve reserve</t>
   </si>
   <si>
-    <t>Minimum founder capital, investment, or available credit needed to avoid dropping below the reserve.</t>
+    <t>Capital required in total, regardless of whether it is founder capital, debt, or investment.</t>
   </si>
   <si>
     <t>Recommended 10% contingency</t>
   </si>
   <si>
-    <t>Buffer for delayed launch collections, refunds, and event/contractor variance.</t>
-  </si>
-  <si>
-    <t>Recommended initial capitalization</t>
-  </si>
-  <si>
-    <t>Base-case cash to commit before launch if launch fees are collected on schedule.</t>
-  </si>
-  <si>
-    <t>Current starting capital assumption</t>
-  </si>
-  <si>
-    <t>Editable Assumptions input.</t>
-  </si>
-  <si>
-    <t>Capital surplus / (shortfall)</t>
-  </si>
-  <si>
-    <t>Positive means the model preserves the reserve; negative means close the gap before launch.</t>
+    <t>Delay/refund/collection-risk buffer.</t>
+  </si>
+  <si>
+    <t>Recommended total committed capital</t>
+  </si>
+  <si>
+    <t>Capital that should be committed or contractually available before launch.</t>
+  </si>
+  <si>
+    <t>Scheduled starting capital and external draws</t>
+  </si>
+  <si>
+    <t>Only enter funded or formally committed sources.</t>
+  </si>
+  <si>
+    <t>Committed capital surplus / (shortfall)</t>
+  </si>
+  <si>
+    <t>Positive means the plan meets the target; negative means reduce burn, accelerate receipts, or close funding.</t>
   </si>
   <si>
     <t>Funding order</t>
@@ -461,34 +455,43 @@
     <t>First</t>
   </si>
   <si>
-    <t>Collect launch fees on milestone-based terms and annual membership revenue upfront where possible.</t>
-  </si>
-  <si>
-    <t>2. Founder capital</t>
-  </si>
-  <si>
-    <t>Base case</t>
-  </si>
-  <si>
-    <t>Use for the calculated reserve requirement and initial legal/product work; it is the cleanest early-stage capital when no recurring cash flow exists.</t>
-  </si>
-  <si>
-    <t>3. Small working-capital line</t>
-  </si>
-  <si>
-    <t>Contingency only</t>
-  </si>
-  <si>
-    <t>Use only for short collection timing gaps after contracts and recurring receipts are demonstrated; do not use it to finance speculative events or open-ended payroll.</t>
-  </si>
-  <si>
-    <t>4. Strategic/equity investment</t>
+    <t>Collect launch fees in milestone-based installments and annual membership revenue upfront where possible.</t>
+  </si>
+  <si>
+    <t>2. Delayable founder draw and staged initial payments</t>
+  </si>
+  <si>
+    <t>Cash preservation</t>
+  </si>
+  <si>
+    <t>Use start-month controls and payment schedules to align cash cost with actual partner/member activation, not with a calendar date.</t>
+  </si>
+  <si>
+    <t>3. Founder capital or committed outside investment</t>
+  </si>
+  <si>
+    <t>Base-case gap</t>
+  </si>
+  <si>
+    <t>Fund the calculated reserve requirement and legal/product milestones. Draw later only if the source is committed before the cash trough.</t>
+  </si>
+  <si>
+    <t>4. Small working-capital line</t>
+  </si>
+  <si>
+    <t>Contingency</t>
+  </si>
+  <si>
+    <t>Use only for contracted timing gaps after recurring collections exist; do not rely on debt for speculative events or open-ended payroll.</t>
+  </si>
+  <si>
+    <t>5. Strategic/equity investment</t>
   </si>
   <si>
     <t>Expansion</t>
   </si>
   <si>
-    <t>Use for multi-market expansion, a dedicated facility, accelerated Connected Garage development, or a staffed partner-success/content team, not to cover an avoidable early operating deficit.</t>
+    <t>Use for multi-market expansion, a facility, accelerated Connected Garage development, or a staffed team.</t>
   </si>
   <si>
     <t>Mature First-Market Annual Run Rate</t>
@@ -521,7 +524,7 @@
     <t>Annual consumer members</t>
   </si>
   <si>
-    <t>At $99 annual dues in the base case.</t>
+    <t>At annual member dues in the base case.</t>
   </si>
   <si>
     <t>Completed bookings / Certified Partner / month</t>
@@ -967,7 +970,7 @@
   <sheetPr>
     <tabColor rgb="FF17324D"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
@@ -1002,14 +1005,6 @@
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1025,18 +1020,18 @@
   <sheetPr>
     <tabColor rgb="FF276678"/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="42.7109375" customWidth="1"/>
+    <col min="1" max="1" width="44.7109375" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" customWidth="1"/>
-    <col min="4" max="4" width="68.7109375" customWidth="1"/>
+    <col min="4" max="4" width="70.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1044,302 +1039,304 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B4" s="6">
         <v>4000</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="7">
+        <v>4</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="B5" s="6">
-        <v>2000</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="6">
+        <v>2000</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="B6" s="6">
-        <v>1500</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="6">
-        <v>1500</v>
+        <v>20</v>
+      </c>
+      <c r="B7" s="7">
+        <v>2</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>22</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D7" s="3"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B8" s="6">
         <v>1500</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="6">
-        <v>1250</v>
+        <v>23</v>
+      </c>
+      <c r="B9" s="7">
+        <v>3</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>26</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D9" s="3"/>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B10" s="6">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B11" s="7">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>31</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D11" s="3"/>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="5" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B12" s="6">
-        <v>25000</v>
+        <v>1500</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="6">
-        <v>10000</v>
+        <v>29</v>
+      </c>
+      <c r="B13" s="7">
+        <v>4</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D13" s="3"/>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="5" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B14" s="6">
-        <v>8000</v>
+        <v>1250</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="3"/>
+        <v>13</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="6">
-        <v>6000</v>
+        <v>32</v>
+      </c>
+      <c r="B15" s="7">
+        <v>4</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="D15" s="3"/>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="5" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B16" s="6">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="3"/>
+        <v>13</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" s="6">
-        <v>2000</v>
+        <v>35</v>
+      </c>
+      <c r="B17" s="7">
+        <v>7</v>
       </c>
       <c r="C17" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="3"/>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="5" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B18" s="6">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="3"/>
+        <v>38</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B19" s="6">
-        <v>6000</v>
+        <v>4000</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B20" s="6">
-        <v>4000</v>
+        <v>1500</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="3"/>
+        <v>41</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" s="6">
+        <v>499</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="6">
-        <v>4000</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>48</v>
-      </c>
+      <c r="D21" s="3"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B22" s="6">
-        <v>1500</v>
+        <v>199</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>50</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="D22" s="3"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B23" s="6">
-        <v>499</v>
+        <v>99</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D23" s="3"/>
+        <v>49</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B24" s="6">
-        <v>199</v>
+        <v>40</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="3"/>
+      <c r="D24" s="3" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B25" s="6">
-        <v>99</v>
+        <v>3000</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>55</v>
@@ -1353,7 +1350,7 @@
         <v>57</v>
       </c>
       <c r="B26" s="6">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>58</v>
@@ -1367,55 +1364,27 @@
         <v>60</v>
       </c>
       <c r="B27" s="6">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" s="6">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="B28" s="6">
-        <v>70000</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B29" s="6">
-        <v>0</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B30" s="6">
-        <v>0</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1431,16 +1400,16 @@
   <sheetPr>
     <tabColor rgb="FF3A7D44"/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="39.7109375" customWidth="1"/>
+    <col min="1" max="1" width="40.7109375" customWidth="1"/>
     <col min="2" max="13" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1457,53 +1426,53 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2" s="8" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="J4" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="L4" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="M4" s="4" t="s">
         <v>78</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="5" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B5" s="7">
         <v>0</v>
@@ -1544,7 +1513,7 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="5" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B6" s="7">
         <v>0</v>
@@ -1585,7 +1554,7 @@
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="5" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B7" s="7">
         <v>0</v>
@@ -1626,7 +1595,7 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="5" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B8" s="7">
         <v>0</v>
@@ -1667,7 +1636,7 @@
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B9" s="7">
         <v>0</v>
@@ -1708,7 +1677,7 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="5" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B10" s="7">
         <v>0</v>
@@ -1749,7 +1718,7 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="5" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B11" s="7">
         <v>0</v>
@@ -1788,867 +1757,831 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12" spans="1:13">
+      <c r="A12" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="6">
+        <v>0</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0</v>
+      </c>
+      <c r="D12" s="6">
+        <v>4000</v>
+      </c>
+      <c r="E12" s="6">
+        <v>6000</v>
+      </c>
+      <c r="F12" s="6">
+        <v>8000</v>
+      </c>
+      <c r="G12" s="6">
+        <v>8000</v>
+      </c>
+      <c r="H12" s="6">
+        <v>2000</v>
+      </c>
+      <c r="I12" s="6">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6">
+        <v>2000</v>
+      </c>
+      <c r="K12" s="6">
+        <v>0</v>
+      </c>
+      <c r="L12" s="6">
+        <v>0</v>
+      </c>
+      <c r="M12" s="6">
+        <v>0</v>
+      </c>
+    </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="2" t="s">
-        <v>92</v>
+      <c r="A13" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="6">
+        <v>0</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0</v>
+      </c>
+      <c r="D13" s="6">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6">
+        <v>0</v>
+      </c>
+      <c r="F13" s="6">
+        <v>5000</v>
+      </c>
+      <c r="G13" s="6">
+        <v>5000</v>
+      </c>
+      <c r="H13" s="6">
+        <v>0</v>
+      </c>
+      <c r="I13" s="6">
+        <v>0</v>
+      </c>
+      <c r="J13" s="6">
+        <v>0</v>
+      </c>
+      <c r="K13" s="6">
+        <v>0</v>
+      </c>
+      <c r="L13" s="6">
+        <v>0</v>
+      </c>
+      <c r="M13" s="6">
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B14" s="9">
-        <f>B5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="9">
-        <f>C5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="9">
-        <f>D5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="9">
-        <f>E5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="F14" s="9">
-        <f>F5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="9">
-        <f>G5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="9">
-        <f>H5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="I14" s="9">
-        <f>I5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="J14" s="9">
-        <f>J5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="K14" s="9">
-        <f>K5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="L14" s="9">
-        <f>L5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-      <c r="M14" s="9">
-        <f>M5*Assumptions!$B$21</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
-      <c r="A15" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B15" s="9">
-        <f>B6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="9">
-        <f>C6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="D15" s="9">
-        <f>D6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="9">
-        <f>E6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="9">
-        <f>F6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="G15" s="9">
-        <f>G6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="9">
-        <f>H6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="9">
-        <f>I6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="9">
-        <f>J6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="K15" s="9">
-        <f>K6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="L15" s="9">
-        <f>L6*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="9">
-        <f>M6*Assumptions!$B$22</f>
+        <v>88</v>
+      </c>
+      <c r="B14" s="6">
+        <v>0</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0</v>
+      </c>
+      <c r="D14" s="6">
+        <v>0</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6">
+        <v>0</v>
+      </c>
+      <c r="I14" s="6">
+        <v>0</v>
+      </c>
+      <c r="J14" s="6">
+        <v>0</v>
+      </c>
+      <c r="K14" s="6">
+        <v>0</v>
+      </c>
+      <c r="L14" s="6">
+        <v>0</v>
+      </c>
+      <c r="M14" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:13">
-      <c r="A16" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="B16" s="9">
-        <f>B7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="C16" s="9">
-        <f>C7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="D16" s="9">
-        <f>D7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="9">
-        <f>E7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="9">
-        <f>F7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="G16" s="9">
-        <f>G7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="9">
-        <f>H7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="I16" s="9">
-        <f>I7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="9">
-        <f>J7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="K16" s="9">
-        <f>K7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="L16" s="9">
-        <f>L7*Assumptions!$B$23</f>
-        <v>0</v>
-      </c>
-      <c r="M16" s="9">
-        <f>M7*Assumptions!$B$23</f>
-        <v>0</v>
+      <c r="A16" s="2" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:13">
       <c r="A17" s="5" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B17" s="9">
-        <f>B8*Assumptions!$B$24</f>
+        <f>B5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="C17" s="9">
-        <f>C8*Assumptions!$B$24</f>
+        <f>C5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="D17" s="9">
-        <f>D8*Assumptions!$B$24</f>
+        <f>D5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="E17" s="9">
-        <f>E8*Assumptions!$B$24</f>
+        <f>E5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="F17" s="9">
-        <f>F8*Assumptions!$B$24</f>
+        <f>F5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="G17" s="9">
-        <f>G8*Assumptions!$B$24</f>
+        <f>G5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="H17" s="9">
-        <f>H8*Assumptions!$B$24</f>
+        <f>H5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="I17" s="9">
-        <f>I8*Assumptions!$B$24</f>
+        <f>I5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <f>J8*Assumptions!$B$24</f>
+        <f>J5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="K17" s="9">
-        <f>K8*Assumptions!$B$24</f>
+        <f>K5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="L17" s="9">
-        <f>L8*Assumptions!$B$24</f>
+        <f>L5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="M17" s="9">
-        <f>M8*Assumptions!$B$24</f>
+        <f>M5*Assumptions!$B$19</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:13">
       <c r="A18" s="5" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B18" s="9">
-        <f>B9*Assumptions!$B$25</f>
+        <f>B6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="C18" s="9">
-        <f>C9*Assumptions!$B$25</f>
+        <f>C6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="D18" s="9">
-        <f>D9*Assumptions!$B$25</f>
+        <f>D6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="E18" s="9">
-        <f>E9*Assumptions!$B$25</f>
+        <f>E6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="F18" s="9">
-        <f>F9*Assumptions!$B$25</f>
+        <f>F6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="G18" s="9">
-        <f>G9*Assumptions!$B$25</f>
+        <f>G6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="H18" s="9">
-        <f>H9*Assumptions!$B$25</f>
+        <f>H6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="I18" s="9">
-        <f>I9*Assumptions!$B$25</f>
+        <f>I6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <f>J9*Assumptions!$B$25</f>
+        <f>J6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="K18" s="9">
-        <f>K9*Assumptions!$B$25</f>
+        <f>K6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="L18" s="9">
-        <f>L9*Assumptions!$B$25</f>
+        <f>L6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
       <c r="M18" s="9">
-        <f>M9*Assumptions!$B$25</f>
+        <f>M6*Assumptions!$B$20</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="5" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B19" s="9">
-        <f>B10*Assumptions!$B$26</f>
+        <f>B7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="C19" s="9">
-        <f>C10*Assumptions!$B$26</f>
+        <f>C7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="D19" s="9">
-        <f>D10*Assumptions!$B$26</f>
+        <f>D7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="E19" s="9">
-        <f>E10*Assumptions!$B$26</f>
+        <f>E7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="F19" s="9">
-        <f>F10*Assumptions!$B$26</f>
+        <f>F7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="G19" s="9">
-        <f>G10*Assumptions!$B$26</f>
+        <f>G7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="H19" s="9">
-        <f>H10*Assumptions!$B$26</f>
+        <f>H7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="I19" s="9">
-        <f>I10*Assumptions!$B$26</f>
+        <f>I7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <f>J10*Assumptions!$B$26</f>
+        <f>J7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="K19" s="9">
-        <f>K10*Assumptions!$B$26</f>
+        <f>K7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="L19" s="9">
-        <f>L10*Assumptions!$B$26</f>
+        <f>L7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
       <c r="M19" s="9">
-        <f>M10*Assumptions!$B$26</f>
+        <f>M7*Assumptions!$B$21</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:13">
       <c r="A20" s="5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B20" s="9">
-        <f>B11*Assumptions!$B$27</f>
+        <f>B8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="C20" s="9">
-        <f>C11*Assumptions!$B$27</f>
+        <f>C8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="D20" s="9">
-        <f>D11*Assumptions!$B$27</f>
+        <f>D8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="E20" s="9">
-        <f>E11*Assumptions!$B$27</f>
+        <f>E8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="F20" s="9">
-        <f>F11*Assumptions!$B$27</f>
+        <f>F8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="G20" s="9">
-        <f>G11*Assumptions!$B$27</f>
+        <f>G8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="H20" s="9">
-        <f>H11*Assumptions!$B$27</f>
+        <f>H8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="I20" s="9">
-        <f>I11*Assumptions!$B$27</f>
+        <f>I8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <f>J11*Assumptions!$B$27</f>
+        <f>J8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="K20" s="9">
-        <f>K11*Assumptions!$B$27</f>
+        <f>K8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="L20" s="9">
-        <f>L11*Assumptions!$B$27</f>
+        <f>L8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
       <c r="M20" s="9">
-        <f>M11*Assumptions!$B$27</f>
+        <f>M8*Assumptions!$B$22</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:13">
       <c r="A21" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>B9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="C21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>C9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="D21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>D9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="E21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>E9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="F21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>F9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="G21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>G9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="H21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>H9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="I21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>I9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>J9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="K21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>K9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="L21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>L9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="M21" s="9">
-        <f>Assumptions!$B$29</f>
+        <f>M9*Assumptions!$B$23</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:13">
       <c r="A22" s="5" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>B10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="C22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>C10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="D22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>D10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="E22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>E10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="F22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>F10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="G22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>G10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="H22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>H10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="I22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>I10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="J22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>J10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="K22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>K10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="L22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>L10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="M22" s="9">
-        <f>Assumptions!$B$30</f>
+        <f>M10*Assumptions!$B$24</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:13">
-      <c r="A23" s="2" t="s">
-        <v>102</v>
+      <c r="A23" s="5" t="s">
+        <v>96</v>
       </c>
       <c r="B23" s="9">
-        <f>SUM(B14:B22)</f>
+        <f>B11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="C23" s="9">
-        <f>SUM(C14:C22)</f>
+        <f>C11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="D23" s="9">
-        <f>SUM(D14:D22)</f>
+        <f>D11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="E23" s="9">
-        <f>SUM(E14:E22)</f>
+        <f>E11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="F23" s="9">
-        <f>SUM(F14:F22)</f>
+        <f>F11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="G23" s="9">
-        <f>SUM(G14:G22)</f>
+        <f>G11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="H23" s="9">
-        <f>SUM(H14:H22)</f>
+        <f>H11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="I23" s="9">
-        <f>SUM(I14:I22)</f>
+        <f>I11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="J23" s="9">
-        <f>SUM(J14:J22)</f>
+        <f>J11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="K23" s="9">
-        <f>SUM(K14:K22)</f>
+        <f>K11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="L23" s="9">
-        <f>SUM(L14:L22)</f>
+        <f>L11*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="M23" s="9">
-        <f>SUM(M14:M22)</f>
+        <f>M11*Assumptions!$B$25</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="A24" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="C24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="J24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="K24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="L24" s="9">
+        <f>Assumptions!$B$28</f>
+        <v>0</v>
+      </c>
+      <c r="M24" s="9">
+        <f>Assumptions!$B$28</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:13">
-      <c r="A25" s="2" t="s">
-        <v>103</v>
+      <c r="A25" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="J25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="K25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="L25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
+      </c>
+      <c r="M25" s="9">
+        <f>Assumptions!$B$29</f>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:13">
-      <c r="A26" s="5" t="s">
-        <v>104</v>
+      <c r="A26" s="2" t="s">
+        <v>99</v>
       </c>
       <c r="B26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(B17:B25)</f>
         <v>0</v>
       </c>
       <c r="C26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(C17:C25)</f>
         <v>0</v>
       </c>
       <c r="D26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(D17:D25)</f>
         <v>0</v>
       </c>
       <c r="E26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(E17:E25)</f>
         <v>0</v>
       </c>
       <c r="F26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(F17:F25)</f>
         <v>0</v>
       </c>
       <c r="G26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(G17:G25)</f>
         <v>0</v>
       </c>
       <c r="H26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(H17:H25)</f>
         <v>0</v>
       </c>
       <c r="I26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(I17:I25)</f>
         <v>0</v>
       </c>
       <c r="J26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(J17:J25)</f>
         <v>0</v>
       </c>
       <c r="K26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(K17:K25)</f>
         <v>0</v>
       </c>
       <c r="L26" s="9">
-        <f>Assumptions!$B$4</f>
+        <f>SUM(L17:L25)</f>
         <v>0</v>
       </c>
       <c r="M26" s="9">
-        <f>Assumptions!$B$4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13">
-      <c r="A27" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="C27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="D27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="E27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="F27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="G27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="H27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="I27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="J27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="K27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="L27" s="9">
-        <f>Assumptions!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="M27" s="9">
-        <f>Assumptions!$B$5</f>
+        <f>SUM(M17:M25)</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:13">
-      <c r="A28" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="B28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="C28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="D28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="E28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="F28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="G28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="H28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="I28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="J28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="K28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="L28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="M28" s="9">
-        <f>Assumptions!$B$6</f>
-        <v>0</v>
+      <c r="A28" s="2" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="29" spans="1:13">
       <c r="A29" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="C29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="D29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="E29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="F29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="G29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="H29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="I29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="J29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="K29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="L29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="M29" s="9">
-        <f>Assumptions!$B$7</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$5,Assumptions!$B$4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:13">
       <c r="A30" s="5" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="C30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="D30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="E30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="F30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="G30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="H30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="I30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="J30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="K30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="L30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
       <c r="M30" s="9">
-        <f>Assumptions!$B$8</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$7,Assumptions!$B$6,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:13">
       <c r="A31" s="5" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="C31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="D31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="E31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="F31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="G31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="H31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="I31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="J31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="K31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="L31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
       <c r="M31" s="9">
-        <f>Assumptions!$B$9</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$9,Assumptions!$B$8,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:13">
       <c r="A32" s="5" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B32" s="9">
         <f>IF(COLUMN()-1&gt;=Assumptions!$B$11,Assumptions!$B$10,0)</f>
@@ -2701,430 +2634,642 @@
     </row>
     <row r="33" spans="1:13">
       <c r="A33" s="5" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="C33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="D33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="E33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="F33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="G33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="H33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="I33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="J33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="K33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="L33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
       <c r="M33" s="9">
-        <f>CHOOSE(COLUMN()-1,Assumptions!$B$13,Assumptions!$B$14,Assumptions!$B$15,Assumptions!$B$16,0,0,0,0,Assumptions!$B$17,0,0,Assumptions!$B$18)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$13,Assumptions!$B$12,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:13">
       <c r="A34" s="5" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="C34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="D34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="E34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="F34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="G34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="H34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="I34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="J34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="K34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="L34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
       <c r="M34" s="9">
-        <f>CHOOSE(COLUMN()-1,0,Assumptions!$B$19,Assumptions!$B$20,0,0,0,0,0,0,0,0,0)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$15,Assumptions!$B$14,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:13">
-      <c r="A35" s="2" t="s">
-        <v>113</v>
+      <c r="A35" s="5" t="s">
+        <v>107</v>
       </c>
       <c r="B35" s="9">
-        <f>SUM(B26:B34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="C35" s="9">
-        <f>SUM(C26:C34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="D35" s="9">
-        <f>SUM(D26:D34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="E35" s="9">
-        <f>SUM(E26:E34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="F35" s="9">
-        <f>SUM(F26:F34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="G35" s="9">
-        <f>SUM(G26:G34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="H35" s="9">
-        <f>SUM(H26:H34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="I35" s="9">
-        <f>SUM(I26:I34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="J35" s="9">
-        <f>SUM(J26:J34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="K35" s="9">
-        <f>SUM(K26:K34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="L35" s="9">
-        <f>SUM(L26:L34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
         <v>0</v>
       </c>
       <c r="M35" s="9">
-        <f>SUM(M26:M34)</f>
+        <f>IF(COLUMN()-1&gt;=Assumptions!$B$17,Assumptions!$B$16,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
+      <c r="A36" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B36" s="9">
+        <f>B12</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="9">
+        <f>C12</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="9">
+        <f>D12</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="9">
+        <f>E12</f>
+        <v>0</v>
+      </c>
+      <c r="F36" s="9">
+        <f>F12</f>
+        <v>0</v>
+      </c>
+      <c r="G36" s="9">
+        <f>G12</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="9">
+        <f>H12</f>
+        <v>0</v>
+      </c>
+      <c r="I36" s="9">
+        <f>I12</f>
+        <v>0</v>
+      </c>
+      <c r="J36" s="9">
+        <f>J12</f>
+        <v>0</v>
+      </c>
+      <c r="K36" s="9">
+        <f>K12</f>
+        <v>0</v>
+      </c>
+      <c r="L36" s="9">
+        <f>L12</f>
+        <v>0</v>
+      </c>
+      <c r="M36" s="9">
+        <f>M12</f>
         <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:13">
-      <c r="A37" s="2" t="s">
-        <v>114</v>
+      <c r="A37" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B37" s="9">
+        <f>B13</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="9">
+        <f>C13</f>
+        <v>0</v>
+      </c>
+      <c r="D37" s="9">
+        <f>D13</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="9">
+        <f>E13</f>
+        <v>0</v>
+      </c>
+      <c r="F37" s="9">
+        <f>F13</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="9">
+        <f>G13</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="9">
+        <f>H13</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="9">
+        <f>I13</f>
+        <v>0</v>
+      </c>
+      <c r="J37" s="9">
+        <f>J13</f>
+        <v>0</v>
+      </c>
+      <c r="K37" s="9">
+        <f>K13</f>
+        <v>0</v>
+      </c>
+      <c r="L37" s="9">
+        <f>L13</f>
+        <v>0</v>
+      </c>
+      <c r="M37" s="9">
+        <f>M13</f>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:13">
-      <c r="A38" s="5" t="s">
-        <v>115</v>
+      <c r="A38" s="2" t="s">
+        <v>110</v>
       </c>
       <c r="B38" s="9">
-        <f>B23-B35</f>
+        <f>SUM(B29:B37)</f>
         <v>0</v>
       </c>
       <c r="C38" s="9">
-        <f>C23-C35</f>
+        <f>SUM(C29:C37)</f>
         <v>0</v>
       </c>
       <c r="D38" s="9">
-        <f>D23-D35</f>
+        <f>SUM(D29:D37)</f>
         <v>0</v>
       </c>
       <c r="E38" s="9">
-        <f>E23-E35</f>
+        <f>SUM(E29:E37)</f>
         <v>0</v>
       </c>
       <c r="F38" s="9">
-        <f>F23-F35</f>
+        <f>SUM(F29:F37)</f>
         <v>0</v>
       </c>
       <c r="G38" s="9">
-        <f>G23-G35</f>
+        <f>SUM(G29:G37)</f>
         <v>0</v>
       </c>
       <c r="H38" s="9">
-        <f>H23-H35</f>
+        <f>SUM(H29:H37)</f>
         <v>0</v>
       </c>
       <c r="I38" s="9">
-        <f>I23-I35</f>
+        <f>SUM(I29:I37)</f>
         <v>0</v>
       </c>
       <c r="J38" s="9">
-        <f>J23-J35</f>
+        <f>SUM(J29:J37)</f>
         <v>0</v>
       </c>
       <c r="K38" s="9">
-        <f>K23-K35</f>
+        <f>SUM(K29:K37)</f>
         <v>0</v>
       </c>
       <c r="L38" s="9">
-        <f>L23-L35</f>
+        <f>SUM(L29:L37)</f>
         <v>0</v>
       </c>
       <c r="M38" s="9">
-        <f>M23-M35</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13">
-      <c r="A39" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="B39" s="9">
-        <f>B38</f>
-        <v>0</v>
-      </c>
-      <c r="C39" s="9">
-        <f>B39+C38</f>
-        <v>0</v>
-      </c>
-      <c r="D39" s="9">
-        <f>C39+D38</f>
-        <v>0</v>
-      </c>
-      <c r="E39" s="9">
-        <f>D39+E38</f>
-        <v>0</v>
-      </c>
-      <c r="F39" s="9">
-        <f>E39+F38</f>
-        <v>0</v>
-      </c>
-      <c r="G39" s="9">
-        <f>F39+G38</f>
-        <v>0</v>
-      </c>
-      <c r="H39" s="9">
-        <f>G39+H38</f>
-        <v>0</v>
-      </c>
-      <c r="I39" s="9">
-        <f>H39+I38</f>
-        <v>0</v>
-      </c>
-      <c r="J39" s="9">
-        <f>I39+J38</f>
-        <v>0</v>
-      </c>
-      <c r="K39" s="9">
-        <f>J39+K38</f>
-        <v>0</v>
-      </c>
-      <c r="L39" s="9">
-        <f>K39+L38</f>
-        <v>0</v>
-      </c>
-      <c r="M39" s="9">
-        <f>L39+M38</f>
+        <f>SUM(M29:M37)</f>
         <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:13">
-      <c r="A40" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B40" s="9">
-        <f>Assumptions!$B$28</f>
-        <v>0</v>
-      </c>
-      <c r="C40" s="9">
-        <f>B41</f>
-        <v>0</v>
-      </c>
-      <c r="D40" s="9">
-        <f>C41</f>
-        <v>0</v>
-      </c>
-      <c r="E40" s="9">
-        <f>D41</f>
-        <v>0</v>
-      </c>
-      <c r="F40" s="9">
-        <f>E41</f>
-        <v>0</v>
-      </c>
-      <c r="G40" s="9">
-        <f>F41</f>
-        <v>0</v>
-      </c>
-      <c r="H40" s="9">
-        <f>G41</f>
-        <v>0</v>
-      </c>
-      <c r="I40" s="9">
-        <f>H41</f>
-        <v>0</v>
-      </c>
-      <c r="J40" s="9">
-        <f>I41</f>
-        <v>0</v>
-      </c>
-      <c r="K40" s="9">
-        <f>J41</f>
-        <v>0</v>
-      </c>
-      <c r="L40" s="9">
-        <f>K41</f>
-        <v>0</v>
-      </c>
-      <c r="M40" s="9">
-        <f>L41</f>
-        <v>0</v>
+      <c r="A40" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="41" spans="1:13">
       <c r="A41" s="5" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B41" s="9">
-        <f>B40+B38</f>
+        <f>B26-B38</f>
         <v>0</v>
       </c>
       <c r="C41" s="9">
-        <f>C40+C38</f>
+        <f>C26-C38</f>
         <v>0</v>
       </c>
       <c r="D41" s="9">
-        <f>D40+D38</f>
+        <f>D26-D38</f>
         <v>0</v>
       </c>
       <c r="E41" s="9">
-        <f>E40+E38</f>
+        <f>E26-E38</f>
         <v>0</v>
       </c>
       <c r="F41" s="9">
-        <f>F40+F38</f>
+        <f>F26-F38</f>
         <v>0</v>
       </c>
       <c r="G41" s="9">
-        <f>G40+G38</f>
+        <f>G26-G38</f>
         <v>0</v>
       </c>
       <c r="H41" s="9">
-        <f>H40+H38</f>
+        <f>H26-H38</f>
         <v>0</v>
       </c>
       <c r="I41" s="9">
-        <f>I40+I38</f>
+        <f>I26-I38</f>
         <v>0</v>
       </c>
       <c r="J41" s="9">
-        <f>J40+J38</f>
+        <f>J26-J38</f>
         <v>0</v>
       </c>
       <c r="K41" s="9">
-        <f>K40+K38</f>
+        <f>K26-K38</f>
         <v>0</v>
       </c>
       <c r="L41" s="9">
-        <f>L40+L38</f>
+        <f>L26-L38</f>
         <v>0</v>
       </c>
       <c r="M41" s="9">
-        <f>M40+M38</f>
+        <f>M26-M38</f>
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:13">
       <c r="A42" s="5" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B42" s="9">
-        <f>B41-Assumptions!$B$12</f>
+        <f>B41</f>
         <v>0</v>
       </c>
       <c r="C42" s="9">
-        <f>C41-Assumptions!$B$12</f>
+        <f>B42+C41</f>
         <v>0</v>
       </c>
       <c r="D42" s="9">
-        <f>D41-Assumptions!$B$12</f>
+        <f>C42+D41</f>
         <v>0</v>
       </c>
       <c r="E42" s="9">
-        <f>E41-Assumptions!$B$12</f>
+        <f>D42+E41</f>
         <v>0</v>
       </c>
       <c r="F42" s="9">
-        <f>F41-Assumptions!$B$12</f>
+        <f>E42+F41</f>
         <v>0</v>
       </c>
       <c r="G42" s="9">
-        <f>G41-Assumptions!$B$12</f>
+        <f>F42+G41</f>
         <v>0</v>
       </c>
       <c r="H42" s="9">
-        <f>H41-Assumptions!$B$12</f>
+        <f>G42+H41</f>
         <v>0</v>
       </c>
       <c r="I42" s="9">
-        <f>I41-Assumptions!$B$12</f>
+        <f>H42+I41</f>
         <v>0</v>
       </c>
       <c r="J42" s="9">
-        <f>J41-Assumptions!$B$12</f>
+        <f>I42+J41</f>
         <v>0</v>
       </c>
       <c r="K42" s="9">
-        <f>K41-Assumptions!$B$12</f>
+        <f>J42+K41</f>
         <v>0</v>
       </c>
       <c r="L42" s="9">
-        <f>L41-Assumptions!$B$12</f>
+        <f>K42+L41</f>
         <v>0</v>
       </c>
       <c r="M42" s="9">
-        <f>M41-Assumptions!$B$12</f>
+        <f>L42+M41</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13">
+      <c r="A43" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B43" s="9">
+        <f>Assumptions!$B$27</f>
+        <v>0</v>
+      </c>
+      <c r="C43" s="9">
+        <f>B45</f>
+        <v>0</v>
+      </c>
+      <c r="D43" s="9">
+        <f>C45</f>
+        <v>0</v>
+      </c>
+      <c r="E43" s="9">
+        <f>D45</f>
+        <v>0</v>
+      </c>
+      <c r="F43" s="9">
+        <f>E45</f>
+        <v>0</v>
+      </c>
+      <c r="G43" s="9">
+        <f>F45</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="9">
+        <f>G45</f>
+        <v>0</v>
+      </c>
+      <c r="I43" s="9">
+        <f>H45</f>
+        <v>0</v>
+      </c>
+      <c r="J43" s="9">
+        <f>I45</f>
+        <v>0</v>
+      </c>
+      <c r="K43" s="9">
+        <f>J45</f>
+        <v>0</v>
+      </c>
+      <c r="L43" s="9">
+        <f>K45</f>
+        <v>0</v>
+      </c>
+      <c r="M43" s="9">
+        <f>L45</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13">
+      <c r="A44" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B44" s="9">
+        <f>B14</f>
+        <v>0</v>
+      </c>
+      <c r="C44" s="9">
+        <f>C14</f>
+        <v>0</v>
+      </c>
+      <c r="D44" s="9">
+        <f>D14</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="9">
+        <f>E14</f>
+        <v>0</v>
+      </c>
+      <c r="F44" s="9">
+        <f>F14</f>
+        <v>0</v>
+      </c>
+      <c r="G44" s="9">
+        <f>G14</f>
+        <v>0</v>
+      </c>
+      <c r="H44" s="9">
+        <f>H14</f>
+        <v>0</v>
+      </c>
+      <c r="I44" s="9">
+        <f>I14</f>
+        <v>0</v>
+      </c>
+      <c r="J44" s="9">
+        <f>J14</f>
+        <v>0</v>
+      </c>
+      <c r="K44" s="9">
+        <f>K14</f>
+        <v>0</v>
+      </c>
+      <c r="L44" s="9">
+        <f>L14</f>
+        <v>0</v>
+      </c>
+      <c r="M44" s="9">
+        <f>M14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13">
+      <c r="A45" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="B45" s="9">
+        <f>B43+B41+B44</f>
+        <v>0</v>
+      </c>
+      <c r="C45" s="9">
+        <f>C43+C41+C44</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="9">
+        <f>D43+D41+D44</f>
+        <v>0</v>
+      </c>
+      <c r="E45" s="9">
+        <f>E43+E41+E44</f>
+        <v>0</v>
+      </c>
+      <c r="F45" s="9">
+        <f>F43+F41+F44</f>
+        <v>0</v>
+      </c>
+      <c r="G45" s="9">
+        <f>G43+G41+G44</f>
+        <v>0</v>
+      </c>
+      <c r="H45" s="9">
+        <f>H43+H41+H44</f>
+        <v>0</v>
+      </c>
+      <c r="I45" s="9">
+        <f>I43+I41+I44</f>
+        <v>0</v>
+      </c>
+      <c r="J45" s="9">
+        <f>J43+J41+J44</f>
+        <v>0</v>
+      </c>
+      <c r="K45" s="9">
+        <f>K43+K41+K44</f>
+        <v>0</v>
+      </c>
+      <c r="L45" s="9">
+        <f>L43+L41+L44</f>
+        <v>0</v>
+      </c>
+      <c r="M45" s="9">
+        <f>M43+M41+M44</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13">
+      <c r="A46" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B46" s="9">
+        <f>B45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="C46" s="9">
+        <f>C45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="9">
+        <f>D45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="E46" s="9">
+        <f>E45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="F46" s="9">
+        <f>F45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="G46" s="9">
+        <f>G45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="9">
+        <f>H45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="I46" s="9">
+        <f>I45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="J46" s="9">
+        <f>J45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="K46" s="9">
+        <f>K45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="L46" s="9">
+        <f>L45-Assumptions!$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="M46" s="9">
+        <f>M45-Assumptions!$B$18</f>
         <v>0</v>
       </c>
     </row>
@@ -3141,199 +3286,210 @@
   <sheetPr>
     <tabColor rgb="FFA65E2E"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="48.7109375" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="50.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
     <col min="3" max="3" width="72.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>121</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B4" s="9">
-        <f>SUM('12 Month Cash Flow'!B23:M23)</f>
+        <f>SUM('12 Month Cash Flow'!B26:M26)</f>
         <v>0</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B5" s="9">
-        <f>SUM('12 Month Cash Flow'!B35:M35)</f>
+        <f>SUM('12 Month Cash Flow'!B38:M38)</f>
         <v>0</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B6" s="9">
         <f>B4-B5</f>
         <v>0</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B7" s="9">
-        <f>MIN('12 Month Cash Flow'!B39:M39)</f>
+        <f>MIN('12 Month Cash Flow'!B42:M42)</f>
         <v>0</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B8" s="9">
-        <f>Assumptions!$B$12</f>
+        <f>Assumptions!$B$18</f>
         <v>0</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B9" s="9">
         <f>MAX(0,-B7+B8)</f>
         <v>0</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B10" s="9">
         <f>B9*10%</f>
         <v>0</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B11" s="9">
         <f>B9+B10</f>
         <v>0</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B12" s="9">
-        <f>Assumptions!$B$28</f>
+        <f>Assumptions!$B$27+SUM('12 Month Cash Flow'!B44:M44)</f>
         <v>0</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B13" s="9">
         <f>B12-B11</f>
         <v>0</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>145</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>148</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>151</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="B20" s="5" t="s">
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="B21" s="5" t="s">
         <v>156</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -3359,222 +3515,222 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B4" s="7">
         <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B5" s="7">
         <v>5</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B6" s="7">
         <v>10</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B7" s="7">
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B8" s="7">
         <v>400</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B9" s="7">
         <v>12</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B10" s="7">
         <v>4</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B13" s="9">
-        <f>B6*Assumptions!$B$21</f>
+        <f>B6*Assumptions!$B$19</f>
         <v>0</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="B14" s="9">
+        <f>B7*Assumptions!$B$20</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>174</v>
-      </c>
-      <c r="B14" s="9">
-        <f>B7*Assumptions!$B$22</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B15" s="9">
-        <f>B4*Assumptions!$B$23*12</f>
+        <f>B4*Assumptions!$B$21*12</f>
         <v>0</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B16" s="9">
-        <f>B5*Assumptions!$B$24*12</f>
+        <f>B5*Assumptions!$B$22*12</f>
         <v>0</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="5" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B17" s="9">
-        <f>B8*Assumptions!$B$25</f>
+        <f>B8*Assumptions!$B$23</f>
         <v>0</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B18" s="9">
-        <f>B4*B9*12*Assumptions!$B$26</f>
+        <f>B4*B9*12*Assumptions!$B$24</f>
         <v>0</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B19" s="9">
-        <f>B10*Assumptions!$B$27</f>
+        <f>B10*Assumptions!$B$25</f>
         <v>0</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B20" s="9">
-        <f>Assumptions!$B$29*12</f>
+        <f>Assumptions!$B$28*12</f>
         <v>0</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="5" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B21" s="9">
-        <f>Assumptions!$B$30*12</f>
+        <f>Assumptions!$B$29*12</f>
         <v>0</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B22" s="9">
         <f>SUM(B13:B21)</f>
         <v>0</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: add vendor campaign delivery costs
</commit_message>
<xml_diff>
--- a/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
+++ b/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Edit yellow cells only. Assumptions controls recurring cost and price drivers; yellow rows on 12 Month Cash Flow control launch timing, one-time payment timing, and outside funding/debt/investment draws. Formula rows recalculate automatically when opened in Excel, Numbers, or Google Sheets.</t>
+          <t>Edit yellow cells only. Assumptions controls recurring cost and price drivers; yellow rows on 12 Month Cash Flow control launch timing, one-time payment timing, and outside funding/debt/investment draws. Vendor campaign contributions are modeled as revenue and their incremental delivery cost is modeled separately. Formula rows recalculate automatically when opened in Excel, Numbers, or Google Sheets.</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44.7109375" customWidth="1" min="1" max="1"/>
@@ -1130,6 +1130,26 @@
       <c r="D33" t="inlineStr">
         <is>
           <t>Months from a partner becoming active before it contributes to booking expectations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Vendor / local campaign delivery cost</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>per campaign</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Total incremental campaign cost: activation staff, permits, media, production, partner materials, and event delivery. Vendor contribution is modeled separately as revenue.</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40.7109375" customWidth="1" min="1" max="1"/>
@@ -2738,394 +2758,450 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Vendor / local campaign delivery cost</t>
+        </is>
+      </c>
+      <c r="B38" s="9">
+        <f>B11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="C38" s="9">
+        <f>C11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="D38" s="9">
+        <f>D11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="E38" s="9">
+        <f>E11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="F38" s="9">
+        <f>F11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="G38" s="9">
+        <f>G11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="H38" s="9">
+        <f>H11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="I38" s="9">
+        <f>I11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="J38" s="9">
+        <f>J11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="K38" s="9">
+        <f>K11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="L38" s="9">
+        <f>L11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+      <c r="M38" s="9">
+        <f>M11*Assumptions!$B$34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="B38" s="9">
-        <f>SUM(B29:B37)</f>
-        <v/>
-      </c>
-      <c r="C38" s="9">
-        <f>SUM(C29:C37)</f>
-        <v/>
-      </c>
-      <c r="D38" s="9">
-        <f>SUM(D29:D37)</f>
-        <v/>
-      </c>
-      <c r="E38" s="9">
-        <f>SUM(E29:E37)</f>
-        <v/>
-      </c>
-      <c r="F38" s="9">
-        <f>SUM(F29:F37)</f>
-        <v/>
-      </c>
-      <c r="G38" s="9">
-        <f>SUM(G29:G37)</f>
-        <v/>
-      </c>
-      <c r="H38" s="9">
-        <f>SUM(H29:H37)</f>
-        <v/>
-      </c>
-      <c r="I38" s="9">
-        <f>SUM(I29:I37)</f>
-        <v/>
-      </c>
-      <c r="J38" s="9">
-        <f>SUM(J29:J37)</f>
-        <v/>
-      </c>
-      <c r="K38" s="9">
-        <f>SUM(K29:K37)</f>
-        <v/>
-      </c>
-      <c r="L38" s="9">
-        <f>SUM(L29:L37)</f>
-        <v/>
-      </c>
-      <c r="M38" s="9">
-        <f>SUM(M29:M37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="B39" s="9">
+        <f>SUM(B29:B38)</f>
+        <v/>
+      </c>
+      <c r="C39" s="9">
+        <f>SUM(C29:C38)</f>
+        <v/>
+      </c>
+      <c r="D39" s="9">
+        <f>SUM(D29:D38)</f>
+        <v/>
+      </c>
+      <c r="E39" s="9">
+        <f>SUM(E29:E38)</f>
+        <v/>
+      </c>
+      <c r="F39" s="9">
+        <f>SUM(F29:F38)</f>
+        <v/>
+      </c>
+      <c r="G39" s="9">
+        <f>SUM(G29:G38)</f>
+        <v/>
+      </c>
+      <c r="H39" s="9">
+        <f>SUM(H29:H38)</f>
+        <v/>
+      </c>
+      <c r="I39" s="9">
+        <f>SUM(I29:I38)</f>
+        <v/>
+      </c>
+      <c r="J39" s="9">
+        <f>SUM(J29:J38)</f>
+        <v/>
+      </c>
+      <c r="K39" s="9">
+        <f>SUM(K29:K38)</f>
+        <v/>
+      </c>
+      <c r="L39" s="9">
+        <f>SUM(L29:L38)</f>
+        <v/>
+      </c>
+      <c r="M39" s="9">
+        <f>SUM(M29:M38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Cash position</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Net operating cash flow</t>
         </is>
       </c>
-      <c r="B41" s="9">
-        <f>B26-B38</f>
-        <v/>
-      </c>
-      <c r="C41" s="9">
-        <f>C26-C38</f>
-        <v/>
-      </c>
-      <c r="D41" s="9">
-        <f>D26-D38</f>
-        <v/>
-      </c>
-      <c r="E41" s="9">
-        <f>E26-E38</f>
-        <v/>
-      </c>
-      <c r="F41" s="9">
-        <f>F26-F38</f>
-        <v/>
-      </c>
-      <c r="G41" s="9">
-        <f>G26-G38</f>
-        <v/>
-      </c>
-      <c r="H41" s="9">
-        <f>H26-H38</f>
-        <v/>
-      </c>
-      <c r="I41" s="9">
-        <f>I26-I38</f>
-        <v/>
-      </c>
-      <c r="J41" s="9">
-        <f>J26-J38</f>
-        <v/>
-      </c>
-      <c r="K41" s="9">
-        <f>K26-K38</f>
-        <v/>
-      </c>
-      <c r="L41" s="9">
-        <f>L26-L38</f>
-        <v/>
-      </c>
-      <c r="M41" s="9">
-        <f>M26-M38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="B42" s="9">
+        <f>B26-B39</f>
+        <v/>
+      </c>
+      <c r="C42" s="9">
+        <f>C26-C39</f>
+        <v/>
+      </c>
+      <c r="D42" s="9">
+        <f>D26-D39</f>
+        <v/>
+      </c>
+      <c r="E42" s="9">
+        <f>E26-E39</f>
+        <v/>
+      </c>
+      <c r="F42" s="9">
+        <f>F26-F39</f>
+        <v/>
+      </c>
+      <c r="G42" s="9">
+        <f>G26-G39</f>
+        <v/>
+      </c>
+      <c r="H42" s="9">
+        <f>H26-H39</f>
+        <v/>
+      </c>
+      <c r="I42" s="9">
+        <f>I26-I39</f>
+        <v/>
+      </c>
+      <c r="J42" s="9">
+        <f>J26-J39</f>
+        <v/>
+      </c>
+      <c r="K42" s="9">
+        <f>K26-K39</f>
+        <v/>
+      </c>
+      <c r="L42" s="9">
+        <f>L26-L39</f>
+        <v/>
+      </c>
+      <c r="M42" s="9">
+        <f>M26-M39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Cumulative cash before funding</t>
         </is>
       </c>
-      <c r="B42" s="9">
-        <f>B41</f>
-        <v/>
-      </c>
-      <c r="C42" s="9">
-        <f>B42+C41</f>
-        <v/>
-      </c>
-      <c r="D42" s="9">
-        <f>C42+D41</f>
-        <v/>
-      </c>
-      <c r="E42" s="9">
-        <f>D42+E41</f>
-        <v/>
-      </c>
-      <c r="F42" s="9">
-        <f>E42+F41</f>
-        <v/>
-      </c>
-      <c r="G42" s="9">
-        <f>F42+G41</f>
-        <v/>
-      </c>
-      <c r="H42" s="9">
-        <f>G42+H41</f>
-        <v/>
-      </c>
-      <c r="I42" s="9">
-        <f>H42+I41</f>
-        <v/>
-      </c>
-      <c r="J42" s="9">
-        <f>I42+J41</f>
-        <v/>
-      </c>
-      <c r="K42" s="9">
-        <f>J42+K41</f>
-        <v/>
-      </c>
-      <c r="L42" s="9">
-        <f>K42+L41</f>
-        <v/>
-      </c>
-      <c r="M42" s="9">
-        <f>L42+M41</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="B43" s="9">
+        <f>B42</f>
+        <v/>
+      </c>
+      <c r="C43" s="9">
+        <f>B43+C42</f>
+        <v/>
+      </c>
+      <c r="D43" s="9">
+        <f>C43+D42</f>
+        <v/>
+      </c>
+      <c r="E43" s="9">
+        <f>D43+E42</f>
+        <v/>
+      </c>
+      <c r="F43" s="9">
+        <f>E43+F42</f>
+        <v/>
+      </c>
+      <c r="G43" s="9">
+        <f>F43+G42</f>
+        <v/>
+      </c>
+      <c r="H43" s="9">
+        <f>G43+H42</f>
+        <v/>
+      </c>
+      <c r="I43" s="9">
+        <f>H43+I42</f>
+        <v/>
+      </c>
+      <c r="J43" s="9">
+        <f>I43+J42</f>
+        <v/>
+      </c>
+      <c r="K43" s="9">
+        <f>J43+K42</f>
+        <v/>
+      </c>
+      <c r="L43" s="9">
+        <f>K43+L42</f>
+        <v/>
+      </c>
+      <c r="M43" s="9">
+        <f>L43+M42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Opening cash</t>
         </is>
       </c>
-      <c r="B43" s="9">
+      <c r="B44" s="9">
         <f>Assumptions!$B$27</f>
         <v/>
       </c>
-      <c r="C43" s="9">
-        <f>B45</f>
-        <v/>
-      </c>
-      <c r="D43" s="9">
-        <f>C45</f>
-        <v/>
-      </c>
-      <c r="E43" s="9">
-        <f>D45</f>
-        <v/>
-      </c>
-      <c r="F43" s="9">
-        <f>E45</f>
-        <v/>
-      </c>
-      <c r="G43" s="9">
-        <f>F45</f>
-        <v/>
-      </c>
-      <c r="H43" s="9">
-        <f>G45</f>
-        <v/>
-      </c>
-      <c r="I43" s="9">
-        <f>H45</f>
-        <v/>
-      </c>
-      <c r="J43" s="9">
-        <f>I45</f>
-        <v/>
-      </c>
-      <c r="K43" s="9">
-        <f>J45</f>
-        <v/>
-      </c>
-      <c r="L43" s="9">
-        <f>K45</f>
-        <v/>
-      </c>
-      <c r="M43" s="9">
-        <f>L45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="C44" s="9">
+        <f>B46</f>
+        <v/>
+      </c>
+      <c r="D44" s="9">
+        <f>C46</f>
+        <v/>
+      </c>
+      <c r="E44" s="9">
+        <f>D46</f>
+        <v/>
+      </c>
+      <c r="F44" s="9">
+        <f>E46</f>
+        <v/>
+      </c>
+      <c r="G44" s="9">
+        <f>F46</f>
+        <v/>
+      </c>
+      <c r="H44" s="9">
+        <f>G46</f>
+        <v/>
+      </c>
+      <c r="I44" s="9">
+        <f>H46</f>
+        <v/>
+      </c>
+      <c r="J44" s="9">
+        <f>I46</f>
+        <v/>
+      </c>
+      <c r="K44" s="9">
+        <f>J46</f>
+        <v/>
+      </c>
+      <c r="L44" s="9">
+        <f>K46</f>
+        <v/>
+      </c>
+      <c r="M44" s="9">
+        <f>L46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>External funding draw</t>
         </is>
       </c>
-      <c r="B44" s="9">
+      <c r="B45" s="9">
         <f>B14</f>
         <v/>
       </c>
-      <c r="C44" s="9">
+      <c r="C45" s="9">
         <f>C14</f>
         <v/>
       </c>
-      <c r="D44" s="9">
+      <c r="D45" s="9">
         <f>D14</f>
         <v/>
       </c>
-      <c r="E44" s="9">
+      <c r="E45" s="9">
         <f>E14</f>
         <v/>
       </c>
-      <c r="F44" s="9">
+      <c r="F45" s="9">
         <f>F14</f>
         <v/>
       </c>
-      <c r="G44" s="9">
+      <c r="G45" s="9">
         <f>G14</f>
         <v/>
       </c>
-      <c r="H44" s="9">
+      <c r="H45" s="9">
         <f>H14</f>
         <v/>
       </c>
-      <c r="I44" s="9">
+      <c r="I45" s="9">
         <f>I14</f>
         <v/>
       </c>
-      <c r="J44" s="9">
+      <c r="J45" s="9">
         <f>J14</f>
         <v/>
       </c>
-      <c r="K44" s="9">
+      <c r="K45" s="9">
         <f>K14</f>
         <v/>
       </c>
-      <c r="L44" s="9">
+      <c r="L45" s="9">
         <f>L14</f>
         <v/>
       </c>
-      <c r="M44" s="9">
+      <c r="M45" s="9">
         <f>M14</f>
         <v/>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Closing cash</t>
         </is>
       </c>
-      <c r="B45" s="9">
-        <f>B43+B41+B44</f>
-        <v/>
-      </c>
-      <c r="C45" s="9">
-        <f>C43+C41+C44</f>
-        <v/>
-      </c>
-      <c r="D45" s="9">
-        <f>D43+D41+D44</f>
-        <v/>
-      </c>
-      <c r="E45" s="9">
-        <f>E43+E41+E44</f>
-        <v/>
-      </c>
-      <c r="F45" s="9">
-        <f>F43+F41+F44</f>
-        <v/>
-      </c>
-      <c r="G45" s="9">
-        <f>G43+G41+G44</f>
-        <v/>
-      </c>
-      <c r="H45" s="9">
-        <f>H43+H41+H44</f>
-        <v/>
-      </c>
-      <c r="I45" s="9">
-        <f>I43+I41+I44</f>
-        <v/>
-      </c>
-      <c r="J45" s="9">
-        <f>J43+J41+J44</f>
-        <v/>
-      </c>
-      <c r="K45" s="9">
-        <f>K43+K41+K44</f>
-        <v/>
-      </c>
-      <c r="L45" s="9">
-        <f>L43+L41+L44</f>
-        <v/>
-      </c>
-      <c r="M45" s="9">
-        <f>M43+M41+M44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="B46" s="9">
+        <f>B44+B42+B45</f>
+        <v/>
+      </c>
+      <c r="C46" s="9">
+        <f>C44+C42+C45</f>
+        <v/>
+      </c>
+      <c r="D46" s="9">
+        <f>D44+D42+D45</f>
+        <v/>
+      </c>
+      <c r="E46" s="9">
+        <f>E44+E42+E45</f>
+        <v/>
+      </c>
+      <c r="F46" s="9">
+        <f>F44+F42+F45</f>
+        <v/>
+      </c>
+      <c r="G46" s="9">
+        <f>G44+G42+G45</f>
+        <v/>
+      </c>
+      <c r="H46" s="9">
+        <f>H44+H42+H45</f>
+        <v/>
+      </c>
+      <c r="I46" s="9">
+        <f>I44+I42+I45</f>
+        <v/>
+      </c>
+      <c r="J46" s="9">
+        <f>J44+J42+J45</f>
+        <v/>
+      </c>
+      <c r="K46" s="9">
+        <f>K44+K42+K45</f>
+        <v/>
+      </c>
+      <c r="L46" s="9">
+        <f>L44+L42+L45</f>
+        <v/>
+      </c>
+      <c r="M46" s="9">
+        <f>M44+M42+M45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Cash above / (below) reserve</t>
         </is>
       </c>
-      <c r="B46" s="9">
-        <f>B45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="C46" s="9">
-        <f>C45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="D46" s="9">
-        <f>D45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="E46" s="9">
-        <f>E45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="F46" s="9">
-        <f>F45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="G46" s="9">
-        <f>G45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="H46" s="9">
-        <f>H45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="I46" s="9">
-        <f>I45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="J46" s="9">
-        <f>J45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="K46" s="9">
-        <f>K45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="L46" s="9">
-        <f>L45-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="M46" s="9">
-        <f>M45-Assumptions!$B$18</f>
+      <c r="B47" s="9">
+        <f>B46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="C47" s="9">
+        <f>C46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="D47" s="9">
+        <f>D46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="E47" s="9">
+        <f>E46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="F47" s="9">
+        <f>F46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="G47" s="9">
+        <f>G46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="H47" s="9">
+        <f>H46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="I47" s="9">
+        <f>I46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="J47" s="9">
+        <f>J46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="K47" s="9">
+        <f>K46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="L47" s="9">
+        <f>L46-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="M47" s="9">
+        <f>M46-Assumptions!$B$18</f>
         <v/>
       </c>
     </row>
@@ -3199,7 +3275,7 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>SUM('12 Month Cash Flow'!B38:M38)</f>
+        <f>SUM('12 Month Cash Flow'!B39:M39)</f>
         <v/>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -3231,7 +3307,7 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>MIN('12 Month Cash Flow'!B42:M42)</f>
+        <f>MIN('12 Month Cash Flow'!B43:M43)</f>
         <v/>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -3311,7 +3387,7 @@
         </is>
       </c>
       <c r="B12" s="9">
-        <f>Assumptions!$B$27+SUM('12 Month Cash Flow'!B44:M44)</f>
+        <f>Assumptions!$B$27+SUM('12 Month Cash Flow'!B45:M45)</f>
         <v/>
       </c>
       <c r="C12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: format booking volume as counts
</commit_message>
<xml_diff>
--- a/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
+++ b/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
@@ -114,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,6 +131,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1072,7 +1073,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
@@ -1477,51 +1477,51 @@
           <t>Completed attributable bookings (formula)</t>
         </is>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="L10" s="9">
+      <c r="L10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
-      <c r="M10" s="9">
+      <c r="M10" s="10">
         <f>IF(COLUMN()-1&lt;=Assumptions!$B$33,0,INDEX($B$7:$M$7,1,COLUMN()-1-Assumptions!$B$33)*Assumptions!$B$32/Assumptions!$B$31)</f>
         <v/>
       </c>
@@ -2867,7 +2867,6 @@
         <v/>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: add new member acquisition costs
</commit_message>
<xml_diff>
--- a/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
+++ b/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
@@ -520,7 +520,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Edit yellow cells only. Assumptions controls recurring cost and price drivers; yellow rows on 12 Month Cash Flow control launch timing, one-time payment timing, and outside funding/debt/investment draws. Vendor campaign contributions are modeled as revenue and their incremental delivery cost is modeled separately. Formula rows recalculate automatically when opened in Excel, Numbers, or Google Sheets.</t>
+          <t>Edit yellow cells only. Assumptions controls recurring cost, member-acquisition cost, and price drivers; yellow rows on 12 Month Cash Flow control launch timing, one-time payment timing, and outside funding/debt/investment draws. Vendor campaign contributions are modeled as revenue and their incremental delivery cost is modeled separately. Formula rows recalculate automatically when opened in Excel, Numbers, or Google Sheets.</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44.7109375" customWidth="1" min="1" max="1"/>
@@ -1150,6 +1150,26 @@
       <c r="D34" t="inlineStr">
         <is>
           <t>Total incremental campaign cost: activation staff, permits, media, production, partner materials, and event delivery. Vendor contribution is modeled separately as revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>New member acquisition / onboarding cost</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>per new annual member</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Paid acquisition, referral credit, onboarding materials, and member-offer cost. Set to zero for an organic-only scenario.</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40.7109375" customWidth="1" min="1" max="1"/>
@@ -2813,394 +2833,450 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>New member acquisition / onboarding cost</t>
+        </is>
+      </c>
+      <c r="B39" s="9">
+        <f>B9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="C39" s="9">
+        <f>C9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="D39" s="9">
+        <f>D9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="E39" s="9">
+        <f>E9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="F39" s="9">
+        <f>F9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="G39" s="9">
+        <f>G9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="H39" s="9">
+        <f>H9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="I39" s="9">
+        <f>I9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="J39" s="9">
+        <f>J9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="K39" s="9">
+        <f>K9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="L39" s="9">
+        <f>L9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+      <c r="M39" s="9">
+        <f>M9*Assumptions!$B$35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="B39" s="9">
-        <f>SUM(B29:B38)</f>
-        <v/>
-      </c>
-      <c r="C39" s="9">
-        <f>SUM(C29:C38)</f>
-        <v/>
-      </c>
-      <c r="D39" s="9">
-        <f>SUM(D29:D38)</f>
-        <v/>
-      </c>
-      <c r="E39" s="9">
-        <f>SUM(E29:E38)</f>
-        <v/>
-      </c>
-      <c r="F39" s="9">
-        <f>SUM(F29:F38)</f>
-        <v/>
-      </c>
-      <c r="G39" s="9">
-        <f>SUM(G29:G38)</f>
-        <v/>
-      </c>
-      <c r="H39" s="9">
-        <f>SUM(H29:H38)</f>
-        <v/>
-      </c>
-      <c r="I39" s="9">
-        <f>SUM(I29:I38)</f>
-        <v/>
-      </c>
-      <c r="J39" s="9">
-        <f>SUM(J29:J38)</f>
-        <v/>
-      </c>
-      <c r="K39" s="9">
-        <f>SUM(K29:K38)</f>
-        <v/>
-      </c>
-      <c r="L39" s="9">
-        <f>SUM(L29:L38)</f>
-        <v/>
-      </c>
-      <c r="M39" s="9">
-        <f>SUM(M29:M38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Cash position</t>
-        </is>
-      </c>
-    </row>
+      <c r="B40" s="9">
+        <f>SUM(B29:B39)</f>
+        <v/>
+      </c>
+      <c r="C40" s="9">
+        <f>SUM(C29:C39)</f>
+        <v/>
+      </c>
+      <c r="D40" s="9">
+        <f>SUM(D29:D39)</f>
+        <v/>
+      </c>
+      <c r="E40" s="9">
+        <f>SUM(E29:E39)</f>
+        <v/>
+      </c>
+      <c r="F40" s="9">
+        <f>SUM(F29:F39)</f>
+        <v/>
+      </c>
+      <c r="G40" s="9">
+        <f>SUM(G29:G39)</f>
+        <v/>
+      </c>
+      <c r="H40" s="9">
+        <f>SUM(H29:H39)</f>
+        <v/>
+      </c>
+      <c r="I40" s="9">
+        <f>SUM(I29:I39)</f>
+        <v/>
+      </c>
+      <c r="J40" s="9">
+        <f>SUM(J29:J39)</f>
+        <v/>
+      </c>
+      <c r="K40" s="9">
+        <f>SUM(K29:K39)</f>
+        <v/>
+      </c>
+      <c r="L40" s="9">
+        <f>SUM(L29:L39)</f>
+        <v/>
+      </c>
+      <c r="M40" s="9">
+        <f>SUM(M29:M39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Net operating cash flow</t>
-        </is>
-      </c>
-      <c r="B42" s="9">
-        <f>B26-B39</f>
-        <v/>
-      </c>
-      <c r="C42" s="9">
-        <f>C26-C39</f>
-        <v/>
-      </c>
-      <c r="D42" s="9">
-        <f>D26-D39</f>
-        <v/>
-      </c>
-      <c r="E42" s="9">
-        <f>E26-E39</f>
-        <v/>
-      </c>
-      <c r="F42" s="9">
-        <f>F26-F39</f>
-        <v/>
-      </c>
-      <c r="G42" s="9">
-        <f>G26-G39</f>
-        <v/>
-      </c>
-      <c r="H42" s="9">
-        <f>H26-H39</f>
-        <v/>
-      </c>
-      <c r="I42" s="9">
-        <f>I26-I39</f>
-        <v/>
-      </c>
-      <c r="J42" s="9">
-        <f>J26-J39</f>
-        <v/>
-      </c>
-      <c r="K42" s="9">
-        <f>K26-K39</f>
-        <v/>
-      </c>
-      <c r="L42" s="9">
-        <f>L26-L39</f>
-        <v/>
-      </c>
-      <c r="M42" s="9">
-        <f>M26-M39</f>
-        <v/>
+          <t>Cash position</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Cumulative cash before funding</t>
+          <t>Net operating cash flow</t>
         </is>
       </c>
       <c r="B43" s="9">
-        <f>B42</f>
+        <f>B26-B40</f>
         <v/>
       </c>
       <c r="C43" s="9">
-        <f>B43+C42</f>
+        <f>C26-C40</f>
         <v/>
       </c>
       <c r="D43" s="9">
-        <f>C43+D42</f>
+        <f>D26-D40</f>
         <v/>
       </c>
       <c r="E43" s="9">
-        <f>D43+E42</f>
+        <f>E26-E40</f>
         <v/>
       </c>
       <c r="F43" s="9">
-        <f>E43+F42</f>
+        <f>F26-F40</f>
         <v/>
       </c>
       <c r="G43" s="9">
-        <f>F43+G42</f>
+        <f>G26-G40</f>
         <v/>
       </c>
       <c r="H43" s="9">
-        <f>G43+H42</f>
+        <f>H26-H40</f>
         <v/>
       </c>
       <c r="I43" s="9">
-        <f>H43+I42</f>
+        <f>I26-I40</f>
         <v/>
       </c>
       <c r="J43" s="9">
-        <f>I43+J42</f>
+        <f>J26-J40</f>
         <v/>
       </c>
       <c r="K43" s="9">
-        <f>J43+K42</f>
+        <f>K26-K40</f>
         <v/>
       </c>
       <c r="L43" s="9">
-        <f>K43+L42</f>
+        <f>L26-L40</f>
         <v/>
       </c>
       <c r="M43" s="9">
-        <f>L43+M42</f>
+        <f>M26-M40</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Opening cash</t>
+          <t>Cumulative cash before funding</t>
         </is>
       </c>
       <c r="B44" s="9">
-        <f>Assumptions!$B$27</f>
+        <f>B43</f>
         <v/>
       </c>
       <c r="C44" s="9">
-        <f>B46</f>
+        <f>B44+C43</f>
         <v/>
       </c>
       <c r="D44" s="9">
-        <f>C46</f>
+        <f>C44+D43</f>
         <v/>
       </c>
       <c r="E44" s="9">
-        <f>D46</f>
+        <f>D44+E43</f>
         <v/>
       </c>
       <c r="F44" s="9">
-        <f>E46</f>
+        <f>E44+F43</f>
         <v/>
       </c>
       <c r="G44" s="9">
-        <f>F46</f>
+        <f>F44+G43</f>
         <v/>
       </c>
       <c r="H44" s="9">
-        <f>G46</f>
+        <f>G44+H43</f>
         <v/>
       </c>
       <c r="I44" s="9">
-        <f>H46</f>
+        <f>H44+I43</f>
         <v/>
       </c>
       <c r="J44" s="9">
-        <f>I46</f>
+        <f>I44+J43</f>
         <v/>
       </c>
       <c r="K44" s="9">
-        <f>J46</f>
+        <f>J44+K43</f>
         <v/>
       </c>
       <c r="L44" s="9">
-        <f>K46</f>
+        <f>K44+L43</f>
         <v/>
       </c>
       <c r="M44" s="9">
-        <f>L46</f>
+        <f>L44+M43</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>External funding draw</t>
+          <t>Opening cash</t>
         </is>
       </c>
       <c r="B45" s="9">
-        <f>B14</f>
+        <f>Assumptions!$B$27</f>
         <v/>
       </c>
       <c r="C45" s="9">
-        <f>C14</f>
+        <f>B47</f>
         <v/>
       </c>
       <c r="D45" s="9">
-        <f>D14</f>
+        <f>C47</f>
         <v/>
       </c>
       <c r="E45" s="9">
-        <f>E14</f>
+        <f>D47</f>
         <v/>
       </c>
       <c r="F45" s="9">
-        <f>F14</f>
+        <f>E47</f>
         <v/>
       </c>
       <c r="G45" s="9">
-        <f>G14</f>
+        <f>F47</f>
         <v/>
       </c>
       <c r="H45" s="9">
-        <f>H14</f>
+        <f>G47</f>
         <v/>
       </c>
       <c r="I45" s="9">
-        <f>I14</f>
+        <f>H47</f>
         <v/>
       </c>
       <c r="J45" s="9">
-        <f>J14</f>
+        <f>I47</f>
         <v/>
       </c>
       <c r="K45" s="9">
-        <f>K14</f>
+        <f>J47</f>
         <v/>
       </c>
       <c r="L45" s="9">
-        <f>L14</f>
+        <f>K47</f>
         <v/>
       </c>
       <c r="M45" s="9">
-        <f>M14</f>
+        <f>L47</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Closing cash</t>
+          <t>External funding draw</t>
         </is>
       </c>
       <c r="B46" s="9">
-        <f>B44+B42+B45</f>
+        <f>B14</f>
         <v/>
       </c>
       <c r="C46" s="9">
-        <f>C44+C42+C45</f>
+        <f>C14</f>
         <v/>
       </c>
       <c r="D46" s="9">
-        <f>D44+D42+D45</f>
+        <f>D14</f>
         <v/>
       </c>
       <c r="E46" s="9">
-        <f>E44+E42+E45</f>
+        <f>E14</f>
         <v/>
       </c>
       <c r="F46" s="9">
-        <f>F44+F42+F45</f>
+        <f>F14</f>
         <v/>
       </c>
       <c r="G46" s="9">
-        <f>G44+G42+G45</f>
+        <f>G14</f>
         <v/>
       </c>
       <c r="H46" s="9">
-        <f>H44+H42+H45</f>
+        <f>H14</f>
         <v/>
       </c>
       <c r="I46" s="9">
-        <f>I44+I42+I45</f>
+        <f>I14</f>
         <v/>
       </c>
       <c r="J46" s="9">
-        <f>J44+J42+J45</f>
+        <f>J14</f>
         <v/>
       </c>
       <c r="K46" s="9">
-        <f>K44+K42+K45</f>
+        <f>K14</f>
         <v/>
       </c>
       <c r="L46" s="9">
-        <f>L44+L42+L45</f>
+        <f>L14</f>
         <v/>
       </c>
       <c r="M46" s="9">
-        <f>M44+M42+M45</f>
+        <f>M14</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>Closing cash</t>
+        </is>
+      </c>
+      <c r="B47" s="9">
+        <f>B45+B43+B46</f>
+        <v/>
+      </c>
+      <c r="C47" s="9">
+        <f>C45+C43+C46</f>
+        <v/>
+      </c>
+      <c r="D47" s="9">
+        <f>D45+D43+D46</f>
+        <v/>
+      </c>
+      <c r="E47" s="9">
+        <f>E45+E43+E46</f>
+        <v/>
+      </c>
+      <c r="F47" s="9">
+        <f>F45+F43+F46</f>
+        <v/>
+      </c>
+      <c r="G47" s="9">
+        <f>G45+G43+G46</f>
+        <v/>
+      </c>
+      <c r="H47" s="9">
+        <f>H45+H43+H46</f>
+        <v/>
+      </c>
+      <c r="I47" s="9">
+        <f>I45+I43+I46</f>
+        <v/>
+      </c>
+      <c r="J47" s="9">
+        <f>J45+J43+J46</f>
+        <v/>
+      </c>
+      <c r="K47" s="9">
+        <f>K45+K43+K46</f>
+        <v/>
+      </c>
+      <c r="L47" s="9">
+        <f>L45+L43+L46</f>
+        <v/>
+      </c>
+      <c r="M47" s="9">
+        <f>M45+M43+M46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
           <t>Cash above / (below) reserve</t>
         </is>
       </c>
-      <c r="B47" s="9">
-        <f>B46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="C47" s="9">
-        <f>C46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="D47" s="9">
-        <f>D46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="E47" s="9">
-        <f>E46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="F47" s="9">
-        <f>F46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="G47" s="9">
-        <f>G46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="H47" s="9">
-        <f>H46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="I47" s="9">
-        <f>I46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="J47" s="9">
-        <f>J46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="K47" s="9">
-        <f>K46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="L47" s="9">
-        <f>L46-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="M47" s="9">
-        <f>M46-Assumptions!$B$18</f>
+      <c r="B48" s="9">
+        <f>B47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="C48" s="9">
+        <f>C47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="D48" s="9">
+        <f>D47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="E48" s="9">
+        <f>E47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="F48" s="9">
+        <f>F47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="G48" s="9">
+        <f>G47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="H48" s="9">
+        <f>H47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="I48" s="9">
+        <f>I47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="J48" s="9">
+        <f>J47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="K48" s="9">
+        <f>K47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="L48" s="9">
+        <f>L47-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="M48" s="9">
+        <f>M47-Assumptions!$B$18</f>
         <v/>
       </c>
     </row>
@@ -3274,7 +3350,7 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>SUM('12 Month Cash Flow'!B39:M39)</f>
+        <f>SUM('12 Month Cash Flow'!B40:M40)</f>
         <v/>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -3306,7 +3382,7 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>MIN('12 Month Cash Flow'!B43:M43)</f>
+        <f>MIN('12 Month Cash Flow'!B44:M44)</f>
         <v/>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -3386,7 +3462,7 @@
         </is>
       </c>
       <c r="B12" s="9">
-        <f>Assumptions!$B$27+SUM('12 Month Cash Flow'!B45:M45)</f>
+        <f>Assumptions!$B$27+SUM('12 Month Cash Flow'!B46:M46)</f>
         <v/>
       </c>
       <c r="C12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: add specialty partner booking revenue
</commit_message>
<xml_diff>
--- a/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
+++ b/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Set each recurring expense start month on Assumptions. Move legal, equipment, and other one-time payments across the yellow schedule on 12 Month Cash Flow. Completed bookings are calculated from active Certified Partners after the configurable qualification delay, using the trailing booking window on Assumptions. Use the yellow External funding draw row only when a loan, investment, or founder contribution is expected to close; do not count an uncommitted source as cash.</t>
+          <t>Set each recurring expense start month on Assumptions. Move legal, equipment, and other one-time payments across the yellow schedule on 12 Month Cash Flow. Certified and specialty/infrastructure booking volumes are calculated separately from their own qualification delays, trailing booking targets, and fixed fees on Assumptions. Use the yellow External funding draw row only when a loan, investment, or founder contribution is expected to close; do not count an uncommitted source as cash.</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44.7109375" customWidth="1" min="1" max="1"/>
@@ -976,7 +976,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Completed-booking fee</t>
+          <t>Certified Partner completed-booking fee</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
@@ -1170,6 +1170,66 @@
       <c r="D35" t="inlineStr">
         <is>
           <t>Paid acquisition, referral credit, onboarding materials, and member-offer cost. Set to zero for an organic-only scenario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Specialty / infrastructure booking qualification delay</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Months from a partner becoming active before it contributes to specialty booking expectations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Completed bookings per qualified specialty / infrastructure partner / window</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>bookings</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Total attributable completed bookings expected from each qualified specialty/infrastructure partner over the measurement window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Specialty / infrastructure completed-booking fee</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>per completed booking</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Fixed fee for attributable specialty/infrastructure work; subject to final legal and attribution review.</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1554,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Completed attributable bookings (formula)</t>
+          <t>Completed Certified Partner bookings (formula)</t>
         </is>
       </c>
       <c r="B10" s="10">
@@ -1718,6 +1778,61 @@
         <v>0</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Completed specialty / infrastructure bookings (formula)</t>
+        </is>
+      </c>
+      <c r="B15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="C15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="D15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="E15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="F15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="G15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="H15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="I15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="J15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="K15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="L15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+      <c r="M15" s="10">
+        <f>IF(COLUMN()-1&lt;=Assumptions!$B$36,0,INDEX($B$8:$M$8,1,COLUMN()-1-Assumptions!$B$36)*Assumptions!$B$37/Assumptions!$B$31)</f>
+        <v/>
+      </c>
+    </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
@@ -2007,51 +2122,51 @@
         </is>
       </c>
       <c r="B22" s="9">
-        <f>B10*Assumptions!$B$24</f>
+        <f>B10*Assumptions!$B$24+B15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="C22" s="9">
-        <f>C10*Assumptions!$B$24</f>
+        <f>C10*Assumptions!$B$24+C15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="D22" s="9">
-        <f>D10*Assumptions!$B$24</f>
+        <f>D10*Assumptions!$B$24+D15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="E22" s="9">
-        <f>E10*Assumptions!$B$24</f>
+        <f>E10*Assumptions!$B$24+E15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="F22" s="9">
-        <f>F10*Assumptions!$B$24</f>
+        <f>F10*Assumptions!$B$24+F15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="G22" s="9">
-        <f>G10*Assumptions!$B$24</f>
+        <f>G10*Assumptions!$B$24+G15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="H22" s="9">
-        <f>H10*Assumptions!$B$24</f>
+        <f>H10*Assumptions!$B$24+H15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="I22" s="9">
-        <f>I10*Assumptions!$B$24</f>
+        <f>I10*Assumptions!$B$24+I15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="J22" s="9">
-        <f>J10*Assumptions!$B$24</f>
+        <f>J10*Assumptions!$B$24+J15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="K22" s="9">
-        <f>K10*Assumptions!$B$24</f>
+        <f>K10*Assumptions!$B$24+K15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="L22" s="9">
-        <f>L10*Assumptions!$B$24</f>
+        <f>L10*Assumptions!$B$24+L15*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="M22" s="9">
-        <f>M10*Assumptions!$B$24</f>
+        <f>M10*Assumptions!$B$24+M15*Assumptions!$B$38</f>
         <v/>
       </c>
     </row>
@@ -2942,7 +3057,6 @@
         <v/>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
@@ -3826,12 +3940,12 @@
         </is>
       </c>
       <c r="B18" s="9">
-        <f>B4*B9/Assumptions!$B$31*12*Assumptions!$B$24</f>
+        <f>B4*Assumptions!$B$32/Assumptions!$B$31*12*Assumptions!$B$24+B5*Assumptions!$B$37/Assumptions!$B$31*12*Assumptions!$B$38</f>
         <v/>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Certified Partners x bookings per trailing window / window months x 12 x completed-booking fee.</t>
+          <t>Certified and specialty/infrastructure booking streams use separate qualified-partner volumes, delays, and fixed fees from Assumptions.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add service mix profitability model
</commit_message>
<xml_diff>
--- a/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
+++ b/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
@@ -11,6 +11,7 @@
     <sheet name="12 Month Cash Flow" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Funding" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Mature Run Rate" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Service Economics" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -19,10 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="$#,##0;[Red]($#,##0)"/>
+    <numFmt numFmtId="165" formatCode="$#,##0"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,8 +57,17 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -86,8 +98,23 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017324D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00276678"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -110,11 +137,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00A6A6A6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +173,25 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4019,4 +4079,540 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="008B5E3C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Service Mix and Partner Contribution Economics</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Yellow cells are inputs. Contribution is revenue less direct technician and parts costs, before shop fixed overhead, taxes, rent, service-advisor cost, and Amped Up fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Global assumptions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Labor billing rate</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>225</v>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Use the shop's effective realized labor rate, not posted rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Loaded technician cost</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>65</v>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Wage, payroll burden, benefits, and other direct technician cost per billed hour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Service type</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Labor hours</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Parts retail</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Parts direct cost</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Mix</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Direct cost</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Contribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Cooling / thermal maintenance</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>75</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F10" s="19">
+        <f>B10*$B$5+C10</f>
+        <v/>
+      </c>
+      <c r="G10" s="19">
+        <f>B10*$B$6+D10</f>
+        <v/>
+      </c>
+      <c r="H10" s="19">
+        <f>F10-G10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Low-voltage battery replacement</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>240</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>170</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F11" s="19">
+        <f>B11*$B$5+C11</f>
+        <v/>
+      </c>
+      <c r="G11" s="19">
+        <f>B11*$B$6+D11</f>
+        <v/>
+      </c>
+      <c r="H11" s="19">
+        <f>F11-G11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Pre-purchase EV inspection</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F12" s="19">
+        <f>B12*$B$5+C12</f>
+        <v/>
+      </c>
+      <c r="G12" s="19">
+        <f>B12*$B$6+D12</f>
+        <v/>
+      </c>
+      <c r="H12" s="19">
+        <f>F12-G12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Annual EV maintenance / inspection</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F13" s="19">
+        <f>B13*$B$5+C13</f>
+        <v/>
+      </c>
+      <c r="G13" s="19">
+        <f>B13*$B$6+D13</f>
+        <v/>
+      </c>
+      <c r="H13" s="19">
+        <f>F13-G13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Suspension repair</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>950</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>650</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F14" s="19">
+        <f>B14*$B$5+C14</f>
+        <v/>
+      </c>
+      <c r="G14" s="19">
+        <f>B14*$B$6+D14</f>
+        <v/>
+      </c>
+      <c r="H14" s="19">
+        <f>F14-G14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Noise identification / diagnostic</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F15" s="19">
+        <f>B15*$B$5+C15</f>
+        <v/>
+      </c>
+      <c r="G15" s="19">
+        <f>B15*$B$6+D15</f>
+        <v/>
+      </c>
+      <c r="H15" s="19">
+        <f>F15-G15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Total mix</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="n"/>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="14" t="n"/>
+      <c r="E17" s="20">
+        <f>SUM(E10:E15)</f>
+        <v/>
+      </c>
+      <c r="F17" s="14" t="n"/>
+      <c r="G17" s="14" t="n"/>
+      <c r="H17" s="14" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Weighted average ticket</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="14" t="n"/>
+      <c r="E18" s="14" t="n"/>
+      <c r="F18" s="19">
+        <f>SUMPRODUCT(E10:E15,F10:F15)</f>
+        <v/>
+      </c>
+      <c r="G18" s="19" t="n"/>
+      <c r="H18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Weighted average direct cost</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="n"/>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+      <c r="E19" s="14" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="19">
+        <f>SUMPRODUCT(E10:E15,G10:G15)</f>
+        <v/>
+      </c>
+      <c r="H19" s="19" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Weighted average contribution per booking</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n"/>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="14" t="n"/>
+      <c r="E20" s="14" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="19" t="n"/>
+      <c r="H20" s="19">
+        <f>SUMPRODUCT(E10:E15,H10:H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Network economics at current assumptions</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="21" t="n"/>
+      <c r="G23" s="21" t="n"/>
+      <c r="H23" s="21" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Certified Partner bookings / two-month window</t>
+        </is>
+      </c>
+      <c r="B24" s="22">
+        <f>Assumptions!$B$32</f>
+        <v/>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>bookings</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Certified Partner booking fee</t>
+        </is>
+      </c>
+      <c r="B25" s="19">
+        <f>Assumptions!$B$24</f>
+        <v/>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>per booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Certified Partner monthly membership</t>
+        </is>
+      </c>
+      <c r="B26" s="19">
+        <f>Assumptions!$B$21</f>
+        <v/>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Certified Partner launch fee</t>
+        </is>
+      </c>
+      <c r="B27" s="19">
+        <f>Assumptions!$B$19</f>
+        <v/>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>one time</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Two-month gross contribution</t>
+        </is>
+      </c>
+      <c r="B28" s="19">
+        <f>B24*$H$20</f>
+        <v/>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>before Amped Up fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Two-month booking fees</t>
+        </is>
+      </c>
+      <c r="B29" s="19">
+        <f>B24*B25</f>
+        <v/>
+      </c>
+      <c r="C29" s="14" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Two-month membership fees</t>
+        </is>
+      </c>
+      <c r="B30" s="19">
+        <f>B26*2</f>
+        <v/>
+      </c>
+      <c r="C30" s="14" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Two-month contribution after recurring Amped Up fees</t>
+        </is>
+      </c>
+      <c r="B31" s="19">
+        <f>B28-B29-B30</f>
+        <v/>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>before launch fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>Active-booking-month payback on launch fee</t>
+        </is>
+      </c>
+      <c r="B32" s="23">
+        <f>B27/(B31/2)</f>
+        <v/>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add partner onboarding delivery costs
</commit_message>
<xml_diff>
--- a/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
+++ b/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
@@ -580,7 +580,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Edit yellow cells only. Assumptions controls recurring cost, member-acquisition cost, and price drivers; yellow rows on 12 Month Cash Flow control launch timing, one-time payment timing, and outside funding/debt/investment draws. Vendor campaign contributions are modeled as revenue and their incremental delivery cost is modeled separately. Formula rows recalculate automatically when opened in Excel, Numbers, or Google Sheets.</t>
+          <t>Edit yellow cells only. Assumptions controls recurring cost, member-acquisition cost, partner-onboarding cost, and price drivers; yellow rows on 12 Month Cash Flow control launch timing, one-time payment timing, and outside funding/debt/investment draws. Vendor campaign contributions are modeled as revenue and their incremental delivery cost is modeled separately. Formula rows recalculate automatically when opened in Excel, Numbers, or Google Sheets.</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44.7109375" customWidth="1" min="1" max="1"/>
@@ -1290,6 +1290,46 @@
       <c r="D38" t="inlineStr">
         <is>
           <t>Fixed fee for attributable specialty/infrastructure work; subject to final legal and attribution review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Full Certified Partner onboarding / delivery cost</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>per new partner</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Cash cost for assessment support, training materials, profile production, launch assets, and initial follow-up. Excludes imputed founder labor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Specialty / infrastructure onboarding / delivery cost</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>per new partner</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Cash cost for streamlined verification, profile production, launch assets, and follow-up. Excludes imputed founder labor.</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40.7109375" customWidth="1" min="1" max="1"/>
@@ -3063,394 +3103,505 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Total operating expenses</t>
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Full Certified Partner onboarding / delivery cost</t>
         </is>
       </c>
       <c r="B40" s="9">
-        <f>SUM(B29:B39)</f>
+        <f>B5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="C40" s="9">
-        <f>SUM(C29:C39)</f>
+        <f>C5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="D40" s="9">
-        <f>SUM(D29:D39)</f>
+        <f>D5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="E40" s="9">
-        <f>SUM(E29:E39)</f>
+        <f>E5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="F40" s="9">
-        <f>SUM(F29:F39)</f>
+        <f>F5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="G40" s="9">
-        <f>SUM(G29:G39)</f>
+        <f>G5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="H40" s="9">
-        <f>SUM(H29:H39)</f>
+        <f>H5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="I40" s="9">
-        <f>SUM(I29:I39)</f>
+        <f>I5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="J40" s="9">
-        <f>SUM(J29:J39)</f>
+        <f>J5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="K40" s="9">
-        <f>SUM(K29:K39)</f>
+        <f>K5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="L40" s="9">
-        <f>SUM(L29:L39)</f>
+        <f>L5*Assumptions!$B$39</f>
         <v/>
       </c>
       <c r="M40" s="9">
-        <f>SUM(M29:M39)</f>
+        <f>M5*Assumptions!$B$39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Specialty / infrastructure onboarding / delivery cost</t>
+        </is>
+      </c>
+      <c r="B41" s="9">
+        <f>B6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="C41" s="9">
+        <f>C6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="D41" s="9">
+        <f>D6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="E41" s="9">
+        <f>E6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="F41" s="9">
+        <f>F6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="G41" s="9">
+        <f>G6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="H41" s="9">
+        <f>H6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="I41" s="9">
+        <f>I6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="J41" s="9">
+        <f>J6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="K41" s="9">
+        <f>K6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="L41" s="9">
+        <f>L6*Assumptions!$B$40</f>
+        <v/>
+      </c>
+      <c r="M41" s="9">
+        <f>M6*Assumptions!$B$40</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Cash position</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Net operating cash flow</t>
-        </is>
-      </c>
-      <c r="B43" s="9">
-        <f>B26-B40</f>
-        <v/>
-      </c>
-      <c r="C43" s="9">
-        <f>C26-C40</f>
-        <v/>
-      </c>
-      <c r="D43" s="9">
-        <f>D26-D40</f>
-        <v/>
-      </c>
-      <c r="E43" s="9">
-        <f>E26-E40</f>
-        <v/>
-      </c>
-      <c r="F43" s="9">
-        <f>F26-F40</f>
-        <v/>
-      </c>
-      <c r="G43" s="9">
-        <f>G26-G40</f>
-        <v/>
-      </c>
-      <c r="H43" s="9">
-        <f>H26-H40</f>
-        <v/>
-      </c>
-      <c r="I43" s="9">
-        <f>I26-I40</f>
-        <v/>
-      </c>
-      <c r="J43" s="9">
-        <f>J26-J40</f>
-        <v/>
-      </c>
-      <c r="K43" s="9">
-        <f>K26-K40</f>
-        <v/>
-      </c>
-      <c r="L43" s="9">
-        <f>L26-L40</f>
-        <v/>
-      </c>
-      <c r="M43" s="9">
-        <f>M26-M40</f>
-        <v/>
-      </c>
-    </row>
+          <t>Total operating expenses</t>
+        </is>
+      </c>
+      <c r="B42" s="9">
+        <f>SUM(B29:B41)</f>
+        <v/>
+      </c>
+      <c r="C42" s="9">
+        <f>SUM(C29:C41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="9">
+        <f>SUM(D29:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="9">
+        <f>SUM(E29:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="9">
+        <f>SUM(F29:F41)</f>
+        <v/>
+      </c>
+      <c r="G42" s="9">
+        <f>SUM(G29:G41)</f>
+        <v/>
+      </c>
+      <c r="H42" s="9">
+        <f>SUM(H29:H41)</f>
+        <v/>
+      </c>
+      <c r="I42" s="9">
+        <f>SUM(I29:I41)</f>
+        <v/>
+      </c>
+      <c r="J42" s="9">
+        <f>SUM(J29:J41)</f>
+        <v/>
+      </c>
+      <c r="K42" s="9">
+        <f>SUM(K29:K41)</f>
+        <v/>
+      </c>
+      <c r="L42" s="9">
+        <f>SUM(L29:L41)</f>
+        <v/>
+      </c>
+      <c r="M42" s="9">
+        <f>SUM(M29:M41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
+          <t>Cash position</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Net operating cash flow</t>
+        </is>
+      </c>
+      <c r="B45" s="9">
+        <f>B26-B42</f>
+        <v/>
+      </c>
+      <c r="C45" s="9">
+        <f>C26-C42</f>
+        <v/>
+      </c>
+      <c r="D45" s="9">
+        <f>D26-D42</f>
+        <v/>
+      </c>
+      <c r="E45" s="9">
+        <f>E26-E42</f>
+        <v/>
+      </c>
+      <c r="F45" s="9">
+        <f>F26-F42</f>
+        <v/>
+      </c>
+      <c r="G45" s="9">
+        <f>G26-G42</f>
+        <v/>
+      </c>
+      <c r="H45" s="9">
+        <f>H26-H42</f>
+        <v/>
+      </c>
+      <c r="I45" s="9">
+        <f>I26-I42</f>
+        <v/>
+      </c>
+      <c r="J45" s="9">
+        <f>J26-J42</f>
+        <v/>
+      </c>
+      <c r="K45" s="9">
+        <f>K26-K42</f>
+        <v/>
+      </c>
+      <c r="L45" s="9">
+        <f>L26-L42</f>
+        <v/>
+      </c>
+      <c r="M45" s="9">
+        <f>M26-M42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>Cumulative cash before funding</t>
         </is>
       </c>
-      <c r="B44" s="9">
-        <f>B43</f>
-        <v/>
-      </c>
-      <c r="C44" s="9">
-        <f>B44+C43</f>
-        <v/>
-      </c>
-      <c r="D44" s="9">
-        <f>C44+D43</f>
-        <v/>
-      </c>
-      <c r="E44" s="9">
-        <f>D44+E43</f>
-        <v/>
-      </c>
-      <c r="F44" s="9">
-        <f>E44+F43</f>
-        <v/>
-      </c>
-      <c r="G44" s="9">
-        <f>F44+G43</f>
-        <v/>
-      </c>
-      <c r="H44" s="9">
-        <f>G44+H43</f>
-        <v/>
-      </c>
-      <c r="I44" s="9">
-        <f>H44+I43</f>
-        <v/>
-      </c>
-      <c r="J44" s="9">
-        <f>I44+J43</f>
-        <v/>
-      </c>
-      <c r="K44" s="9">
-        <f>J44+K43</f>
-        <v/>
-      </c>
-      <c r="L44" s="9">
-        <f>K44+L43</f>
-        <v/>
-      </c>
-      <c r="M44" s="9">
-        <f>L44+M43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="B46" s="9">
+        <f>B45</f>
+        <v/>
+      </c>
+      <c r="C46" s="9">
+        <f>B46+C45</f>
+        <v/>
+      </c>
+      <c r="D46" s="9">
+        <f>C46+D45</f>
+        <v/>
+      </c>
+      <c r="E46" s="9">
+        <f>D46+E45</f>
+        <v/>
+      </c>
+      <c r="F46" s="9">
+        <f>E46+F45</f>
+        <v/>
+      </c>
+      <c r="G46" s="9">
+        <f>F46+G45</f>
+        <v/>
+      </c>
+      <c r="H46" s="9">
+        <f>G46+H45</f>
+        <v/>
+      </c>
+      <c r="I46" s="9">
+        <f>H46+I45</f>
+        <v/>
+      </c>
+      <c r="J46" s="9">
+        <f>I46+J45</f>
+        <v/>
+      </c>
+      <c r="K46" s="9">
+        <f>J46+K45</f>
+        <v/>
+      </c>
+      <c r="L46" s="9">
+        <f>K46+L45</f>
+        <v/>
+      </c>
+      <c r="M46" s="9">
+        <f>L46+M45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Opening cash</t>
         </is>
       </c>
-      <c r="B45" s="9">
+      <c r="B47" s="9">
         <f>Assumptions!$B$27</f>
         <v/>
       </c>
-      <c r="C45" s="9">
-        <f>B47</f>
-        <v/>
-      </c>
-      <c r="D45" s="9">
-        <f>C47</f>
-        <v/>
-      </c>
-      <c r="E45" s="9">
-        <f>D47</f>
-        <v/>
-      </c>
-      <c r="F45" s="9">
-        <f>E47</f>
-        <v/>
-      </c>
-      <c r="G45" s="9">
-        <f>F47</f>
-        <v/>
-      </c>
-      <c r="H45" s="9">
-        <f>G47</f>
-        <v/>
-      </c>
-      <c r="I45" s="9">
-        <f>H47</f>
-        <v/>
-      </c>
-      <c r="J45" s="9">
-        <f>I47</f>
-        <v/>
-      </c>
-      <c r="K45" s="9">
-        <f>J47</f>
-        <v/>
-      </c>
-      <c r="L45" s="9">
-        <f>K47</f>
-        <v/>
-      </c>
-      <c r="M45" s="9">
-        <f>L47</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="C47" s="9">
+        <f>B49</f>
+        <v/>
+      </c>
+      <c r="D47" s="9">
+        <f>C49</f>
+        <v/>
+      </c>
+      <c r="E47" s="9">
+        <f>D49</f>
+        <v/>
+      </c>
+      <c r="F47" s="9">
+        <f>E49</f>
+        <v/>
+      </c>
+      <c r="G47" s="9">
+        <f>F49</f>
+        <v/>
+      </c>
+      <c r="H47" s="9">
+        <f>G49</f>
+        <v/>
+      </c>
+      <c r="I47" s="9">
+        <f>H49</f>
+        <v/>
+      </c>
+      <c r="J47" s="9">
+        <f>I49</f>
+        <v/>
+      </c>
+      <c r="K47" s="9">
+        <f>J49</f>
+        <v/>
+      </c>
+      <c r="L47" s="9">
+        <f>K49</f>
+        <v/>
+      </c>
+      <c r="M47" s="9">
+        <f>L49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>External funding draw</t>
         </is>
       </c>
-      <c r="B46" s="9">
+      <c r="B48" s="9">
         <f>B14</f>
         <v/>
       </c>
-      <c r="C46" s="9">
+      <c r="C48" s="9">
         <f>C14</f>
         <v/>
       </c>
-      <c r="D46" s="9">
+      <c r="D48" s="9">
         <f>D14</f>
         <v/>
       </c>
-      <c r="E46" s="9">
+      <c r="E48" s="9">
         <f>E14</f>
         <v/>
       </c>
-      <c r="F46" s="9">
+      <c r="F48" s="9">
         <f>F14</f>
         <v/>
       </c>
-      <c r="G46" s="9">
+      <c r="G48" s="9">
         <f>G14</f>
         <v/>
       </c>
-      <c r="H46" s="9">
+      <c r="H48" s="9">
         <f>H14</f>
         <v/>
       </c>
-      <c r="I46" s="9">
+      <c r="I48" s="9">
         <f>I14</f>
         <v/>
       </c>
-      <c r="J46" s="9">
+      <c r="J48" s="9">
         <f>J14</f>
         <v/>
       </c>
-      <c r="K46" s="9">
+      <c r="K48" s="9">
         <f>K14</f>
         <v/>
       </c>
-      <c r="L46" s="9">
+      <c r="L48" s="9">
         <f>L14</f>
         <v/>
       </c>
-      <c r="M46" s="9">
+      <c r="M48" s="9">
         <f>M14</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Closing cash</t>
         </is>
       </c>
-      <c r="B47" s="9">
-        <f>B45+B43+B46</f>
-        <v/>
-      </c>
-      <c r="C47" s="9">
-        <f>C45+C43+C46</f>
-        <v/>
-      </c>
-      <c r="D47" s="9">
-        <f>D45+D43+D46</f>
-        <v/>
-      </c>
-      <c r="E47" s="9">
-        <f>E45+E43+E46</f>
-        <v/>
-      </c>
-      <c r="F47" s="9">
-        <f>F45+F43+F46</f>
-        <v/>
-      </c>
-      <c r="G47" s="9">
-        <f>G45+G43+G46</f>
-        <v/>
-      </c>
-      <c r="H47" s="9">
-        <f>H45+H43+H46</f>
-        <v/>
-      </c>
-      <c r="I47" s="9">
-        <f>I45+I43+I46</f>
-        <v/>
-      </c>
-      <c r="J47" s="9">
-        <f>J45+J43+J46</f>
-        <v/>
-      </c>
-      <c r="K47" s="9">
-        <f>K45+K43+K46</f>
-        <v/>
-      </c>
-      <c r="L47" s="9">
-        <f>L45+L43+L46</f>
-        <v/>
-      </c>
-      <c r="M47" s="9">
-        <f>M45+M43+M46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="B49" s="9">
+        <f>B47+B45+B48</f>
+        <v/>
+      </c>
+      <c r="C49" s="9">
+        <f>C47+C45+C48</f>
+        <v/>
+      </c>
+      <c r="D49" s="9">
+        <f>D47+D45+D48</f>
+        <v/>
+      </c>
+      <c r="E49" s="9">
+        <f>E47+E45+E48</f>
+        <v/>
+      </c>
+      <c r="F49" s="9">
+        <f>F47+F45+F48</f>
+        <v/>
+      </c>
+      <c r="G49" s="9">
+        <f>G47+G45+G48</f>
+        <v/>
+      </c>
+      <c r="H49" s="9">
+        <f>H47+H45+H48</f>
+        <v/>
+      </c>
+      <c r="I49" s="9">
+        <f>I47+I45+I48</f>
+        <v/>
+      </c>
+      <c r="J49" s="9">
+        <f>J47+J45+J48</f>
+        <v/>
+      </c>
+      <c r="K49" s="9">
+        <f>K47+K45+K48</f>
+        <v/>
+      </c>
+      <c r="L49" s="9">
+        <f>L47+L45+L48</f>
+        <v/>
+      </c>
+      <c r="M49" s="9">
+        <f>M47+M45+M48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Cash above / (below) reserve</t>
         </is>
       </c>
-      <c r="B48" s="9">
-        <f>B47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="C48" s="9">
-        <f>C47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="D48" s="9">
-        <f>D47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="E48" s="9">
-        <f>E47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="F48" s="9">
-        <f>F47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="G48" s="9">
-        <f>G47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="H48" s="9">
-        <f>H47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="I48" s="9">
-        <f>I47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="J48" s="9">
-        <f>J47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="K48" s="9">
-        <f>K47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="L48" s="9">
-        <f>L47-Assumptions!$B$18</f>
-        <v/>
-      </c>
-      <c r="M48" s="9">
-        <f>M47-Assumptions!$B$18</f>
+      <c r="B50" s="9">
+        <f>B49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="C50" s="9">
+        <f>C49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="D50" s="9">
+        <f>D49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="E50" s="9">
+        <f>E49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="F50" s="9">
+        <f>F49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="G50" s="9">
+        <f>G49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="H50" s="9">
+        <f>H49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="I50" s="9">
+        <f>I49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="J50" s="9">
+        <f>J49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="K50" s="9">
+        <f>K49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="L50" s="9">
+        <f>L49-Assumptions!$B$18</f>
+        <v/>
+      </c>
+      <c r="M50" s="9">
+        <f>M49-Assumptions!$B$18</f>
         <v/>
       </c>
     </row>
@@ -3524,7 +3675,7 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>SUM('12 Month Cash Flow'!B40:M40)</f>
+        <f>SUM('12 Month Cash Flow'!B42:M42)</f>
         <v/>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -3556,7 +3707,7 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>MIN('12 Month Cash Flow'!B44:M44)</f>
+        <f>MIN('12 Month Cash Flow'!B46:M46)</f>
         <v/>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -3636,7 +3787,7 @@
         </is>
       </c>
       <c r="B12" s="9">
-        <f>Assumptions!$B$27+SUM('12 Month Cash Flow'!B46:M46)</f>
+        <f>Assumptions!$B$27+SUM('12 Month Cash Flow'!B48:M48)</f>
         <v/>
       </c>
       <c r="C12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: add directory validation phase
</commit_message>
<xml_diff>
--- a/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
+++ b/docs/AMPED_UP_NETWORK_FINANCIAL_MODEL.xlsx
@@ -9,9 +9,10 @@
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="12 Month Cash Flow" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Funding" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Mature Run Rate" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Service Economics" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="6 Month Validation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Funding" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Mature Run Rate" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Service Economics" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -155,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -192,6 +193,8 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -580,7 +583,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Edit yellow cells only. Assumptions controls recurring cost, member-acquisition cost, partner-onboarding cost, and price drivers; yellow rows on 12 Month Cash Flow control launch timing, one-time payment timing, and outside funding/debt/investment draws. Vendor campaign contributions are modeled as revenue and their incremental delivery cost is modeled separately. Formula rows recalculate automatically when opened in Excel, Numbers, or Google Sheets.</t>
+          <t>Edit yellow cells only. Assumptions controls recurring cost, member-acquisition cost, partner-onboarding cost, and price drivers; yellow rows on 12 Month Cash Flow control launch timing, one-time payment timing, and outside funding/debt/investment draws. The 6 Month Validation sheet separately models the directory-and-community phase before paid shop partnerships, including $99 founding memberships and paid expert opportunities. Vendor campaign contributions are modeled as revenue and their incremental delivery cost is modeled separately. Formula rows recalculate automatically when opened in Excel, Numbers, or Google Sheets.</t>
         </is>
       </c>
     </row>
@@ -592,7 +595,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Set each recurring expense start month on Assumptions. Move legal, equipment, and other one-time payments across the yellow schedule on 12 Month Cash Flow. Certified and specialty/infrastructure booking volumes are calculated separately from their own qualification delays, trailing booking targets, and fixed fees on Assumptions. Use the yellow External funding draw row only when a loan, investment, or founder contribution is expected to close; do not count an uncommitted source as cash.</t>
+          <t>Use 6 Month Validation to set the pre-partner membership, expert, product, content, legal, directory-quality, and marketing assumptions. Its founder draw defaults to zero and should remain zero until the paid partner rollout. Set recurring expense start months on Assumptions for the partner rollout. Move legal, equipment, and other one-time payments across the yellow schedule on 12 Month Cash Flow. Certified and specialty/infrastructure booking volumes are calculated separately from their own qualification delays, trailing booking targets, and fixed fees on Assumptions. Use the yellow External funding draw row only when a loan, investment, or founder contribution is expected to close; do not count an uncommitted source as cash.</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3270,6 @@
         <v/>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
@@ -3614,6 +3616,1164 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="004F6D7A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="43" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Six-Month Directory and Community Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Pre-partner demand-validation scenario. No paid shop memberships, launch fees, booking fees, or certification revenue are assumed. Yellow cells are editable inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Validation-phase assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Founding early-access annual membership</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>99</v>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>per member</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Discount/community/issue-tracker access only; do not promise certification, shop availability, or partner benefits that are not live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Paid expert opportunity price</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>59</v>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>per opportunity</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Owner-paid, bounded educational guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Expert payout</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>35</v>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>per completed opportunity</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Paid to a verified community expert/shop after quality/acceptance rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Directory/profile QA cost</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>500</v>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>per month</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Listing research, claim/correction handling, profile quality, and local service taxonomy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Early-access marketing cost</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>500</v>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>per month</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Small content, creator, referral, and community tests; no large paid-media campaign.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Validation reserve</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>cash balance</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Minimum cash buffer during the no-paid-partner phase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Monthly validation ramp</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="n"/>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="21" t="n"/>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="21" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Driver / Cash Flow</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>Month 1</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="inlineStr">
+        <is>
+          <t>Month 2</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>Month 3</t>
+        </is>
+      </c>
+      <c r="E13" s="25" t="inlineStr">
+        <is>
+          <t>Month 4</t>
+        </is>
+      </c>
+      <c r="F13" s="25" t="inlineStr">
+        <is>
+          <t>Month 5</t>
+        </is>
+      </c>
+      <c r="G13" s="25" t="inlineStr">
+        <is>
+          <t>Month 6</t>
+        </is>
+      </c>
+      <c r="H13" s="25" t="inlineStr">
+        <is>
+          <t>Six-month total</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>New founding early-access members</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="H14" s="14">
+        <f>SUM(B14:G14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Completed paid expert opportunities</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="H15" s="14">
+        <f>SUM(B15:G15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Founder draw</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="19">
+        <f>SUM(B16:G16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Engineering / product</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H17" s="19">
+        <f>SUM(B17:G17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Content / social production</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H18" s="19">
+        <f>SUM(B18:G18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Software / payments / data</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F19" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G19" s="15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H19" s="19">
+        <f>SUM(B19:G19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Legal / compliance</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H20" s="19">
+        <f>SUM(B20:G20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Equipment / initial production</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F21" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="19">
+        <f>SUM(B21:G21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="21" t="n"/>
+      <c r="G23" s="21" t="n"/>
+      <c r="H23" s="21" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Founding early-access memberships</t>
+        </is>
+      </c>
+      <c r="B24" s="19">
+        <f>B14*$B$5</f>
+        <v/>
+      </c>
+      <c r="C24" s="19">
+        <f>C14*$B$5</f>
+        <v/>
+      </c>
+      <c r="D24" s="19">
+        <f>D14*$B$5</f>
+        <v/>
+      </c>
+      <c r="E24" s="19">
+        <f>E14*$B$5</f>
+        <v/>
+      </c>
+      <c r="F24" s="19">
+        <f>F14*$B$5</f>
+        <v/>
+      </c>
+      <c r="G24" s="19">
+        <f>G14*$B$5</f>
+        <v/>
+      </c>
+      <c r="H24" s="19">
+        <f>SUM(B24:G24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Paid expert opportunity revenue</t>
+        </is>
+      </c>
+      <c r="B25" s="19">
+        <f>B15*$B$6</f>
+        <v/>
+      </c>
+      <c r="C25" s="19">
+        <f>C15*$B$6</f>
+        <v/>
+      </c>
+      <c r="D25" s="19">
+        <f>D15*$B$6</f>
+        <v/>
+      </c>
+      <c r="E25" s="19">
+        <f>E15*$B$6</f>
+        <v/>
+      </c>
+      <c r="F25" s="19">
+        <f>F15*$B$6</f>
+        <v/>
+      </c>
+      <c r="G25" s="19">
+        <f>G15*$B$6</f>
+        <v/>
+      </c>
+      <c r="H25" s="19">
+        <f>SUM(B25:G25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Total validation revenue</t>
+        </is>
+      </c>
+      <c r="B26" s="19">
+        <f>SUM(B24:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="19">
+        <f>SUM(C24:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="19">
+        <f>SUM(D24:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="19">
+        <f>SUM(E24:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="19">
+        <f>SUM(F24:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="19">
+        <f>SUM(G24:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="19">
+        <f>SUM(H24:H25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Cash costs</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="21" t="n"/>
+      <c r="F28" s="21" t="n"/>
+      <c r="G28" s="21" t="n"/>
+      <c r="H28" s="21" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Founder draw</t>
+        </is>
+      </c>
+      <c r="B29" s="19">
+        <f>B16</f>
+        <v/>
+      </c>
+      <c r="C29" s="19">
+        <f>C16</f>
+        <v/>
+      </c>
+      <c r="D29" s="19">
+        <f>D16</f>
+        <v/>
+      </c>
+      <c r="E29" s="19">
+        <f>E16</f>
+        <v/>
+      </c>
+      <c r="F29" s="19">
+        <f>F16</f>
+        <v/>
+      </c>
+      <c r="G29" s="19">
+        <f>G16</f>
+        <v/>
+      </c>
+      <c r="H29" s="19">
+        <f>SUM(B29:G29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Engineering / product</t>
+        </is>
+      </c>
+      <c r="B30" s="19">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="C30" s="19">
+        <f>C17</f>
+        <v/>
+      </c>
+      <c r="D30" s="19">
+        <f>D17</f>
+        <v/>
+      </c>
+      <c r="E30" s="19">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="F30" s="19">
+        <f>F17</f>
+        <v/>
+      </c>
+      <c r="G30" s="19">
+        <f>G17</f>
+        <v/>
+      </c>
+      <c r="H30" s="19">
+        <f>SUM(B30:G30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Content / social production</t>
+        </is>
+      </c>
+      <c r="B31" s="19">
+        <f>B18</f>
+        <v/>
+      </c>
+      <c r="C31" s="19">
+        <f>C18</f>
+        <v/>
+      </c>
+      <c r="D31" s="19">
+        <f>D18</f>
+        <v/>
+      </c>
+      <c r="E31" s="19">
+        <f>E18</f>
+        <v/>
+      </c>
+      <c r="F31" s="19">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="G31" s="19">
+        <f>G18</f>
+        <v/>
+      </c>
+      <c r="H31" s="19">
+        <f>SUM(B31:G31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>Software / payments / data</t>
+        </is>
+      </c>
+      <c r="B32" s="19">
+        <f>B19</f>
+        <v/>
+      </c>
+      <c r="C32" s="19">
+        <f>C19</f>
+        <v/>
+      </c>
+      <c r="D32" s="19">
+        <f>D19</f>
+        <v/>
+      </c>
+      <c r="E32" s="19">
+        <f>E19</f>
+        <v/>
+      </c>
+      <c r="F32" s="19">
+        <f>F19</f>
+        <v/>
+      </c>
+      <c r="G32" s="19">
+        <f>G19</f>
+        <v/>
+      </c>
+      <c r="H32" s="19">
+        <f>SUM(B32:G32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>Legal / compliance</t>
+        </is>
+      </c>
+      <c r="B33" s="19">
+        <f>B20</f>
+        <v/>
+      </c>
+      <c r="C33" s="19">
+        <f>C20</f>
+        <v/>
+      </c>
+      <c r="D33" s="19">
+        <f>D20</f>
+        <v/>
+      </c>
+      <c r="E33" s="19">
+        <f>E20</f>
+        <v/>
+      </c>
+      <c r="F33" s="19">
+        <f>F20</f>
+        <v/>
+      </c>
+      <c r="G33" s="19">
+        <f>G20</f>
+        <v/>
+      </c>
+      <c r="H33" s="19">
+        <f>SUM(B33:G33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>Equipment / initial production</t>
+        </is>
+      </c>
+      <c r="B34" s="19">
+        <f>B21</f>
+        <v/>
+      </c>
+      <c r="C34" s="19">
+        <f>C21</f>
+        <v/>
+      </c>
+      <c r="D34" s="19">
+        <f>D21</f>
+        <v/>
+      </c>
+      <c r="E34" s="19">
+        <f>E21</f>
+        <v/>
+      </c>
+      <c r="F34" s="19">
+        <f>F21</f>
+        <v/>
+      </c>
+      <c r="G34" s="19">
+        <f>G21</f>
+        <v/>
+      </c>
+      <c r="H34" s="19">
+        <f>SUM(B34:G34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>Directory/profile QA</t>
+        </is>
+      </c>
+      <c r="B35" s="19">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="C35" s="19">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="D35" s="19">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="E35" s="19">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="F35" s="19">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="G35" s="19">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="H35" s="19">
+        <f>SUM(B35:G35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>Early-access marketing</t>
+        </is>
+      </c>
+      <c r="B36" s="19">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="C36" s="19">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="D36" s="19">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="E36" s="19">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="F36" s="19">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="G36" s="19">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="H36" s="19">
+        <f>SUM(B36:G36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>Expert payouts</t>
+        </is>
+      </c>
+      <c r="B37" s="19">
+        <f>B15*$B$7</f>
+        <v/>
+      </c>
+      <c r="C37" s="19">
+        <f>C15*$B$7</f>
+        <v/>
+      </c>
+      <c r="D37" s="19">
+        <f>D15*$B$7</f>
+        <v/>
+      </c>
+      <c r="E37" s="19">
+        <f>E15*$B$7</f>
+        <v/>
+      </c>
+      <c r="F37" s="19">
+        <f>F15*$B$7</f>
+        <v/>
+      </c>
+      <c r="G37" s="19">
+        <f>G15*$B$7</f>
+        <v/>
+      </c>
+      <c r="H37" s="19">
+        <f>SUM(B37:G37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Total validation costs</t>
+        </is>
+      </c>
+      <c r="B38" s="19">
+        <f>SUM(B29:B37)</f>
+        <v/>
+      </c>
+      <c r="C38" s="19">
+        <f>SUM(C29:C37)</f>
+        <v/>
+      </c>
+      <c r="D38" s="19">
+        <f>SUM(D29:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="19">
+        <f>SUM(E29:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="19">
+        <f>SUM(F29:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="19">
+        <f>SUM(G29:G37)</f>
+        <v/>
+      </c>
+      <c r="H38" s="19">
+        <f>SUM(H29:H37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>Cash position</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="n"/>
+      <c r="C40" s="21" t="n"/>
+      <c r="D40" s="21" t="n"/>
+      <c r="E40" s="21" t="n"/>
+      <c r="F40" s="21" t="n"/>
+      <c r="G40" s="21" t="n"/>
+      <c r="H40" s="21" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>Net validation cash flow</t>
+        </is>
+      </c>
+      <c r="B41" s="19">
+        <f>B26-B38</f>
+        <v/>
+      </c>
+      <c r="C41" s="19">
+        <f>C26-C38</f>
+        <v/>
+      </c>
+      <c r="D41" s="19">
+        <f>D26-D38</f>
+        <v/>
+      </c>
+      <c r="E41" s="19">
+        <f>E26-E38</f>
+        <v/>
+      </c>
+      <c r="F41" s="19">
+        <f>F26-F38</f>
+        <v/>
+      </c>
+      <c r="G41" s="19">
+        <f>G26-G38</f>
+        <v/>
+      </c>
+      <c r="H41" s="19">
+        <f>SUM(B41:G41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>Cumulative cash before funding</t>
+        </is>
+      </c>
+      <c r="B42" s="19">
+        <f>B41</f>
+        <v/>
+      </c>
+      <c r="C42" s="19">
+        <f>B42+C41</f>
+        <v/>
+      </c>
+      <c r="D42" s="19">
+        <f>C42+D41</f>
+        <v/>
+      </c>
+      <c r="E42" s="19">
+        <f>D42+E41</f>
+        <v/>
+      </c>
+      <c r="F42" s="19">
+        <f>E42+F41</f>
+        <v/>
+      </c>
+      <c r="G42" s="19">
+        <f>F42+G41</f>
+        <v/>
+      </c>
+      <c r="H42" s="19">
+        <f>SUM(B42:G42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>External funding draw</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="19">
+        <f>SUM(B43:G43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>Closing cash</t>
+        </is>
+      </c>
+      <c r="B44" s="19">
+        <f>B42+B43</f>
+        <v/>
+      </c>
+      <c r="C44" s="19">
+        <f>C42+C43</f>
+        <v/>
+      </c>
+      <c r="D44" s="19">
+        <f>D42+D43</f>
+        <v/>
+      </c>
+      <c r="E44" s="19">
+        <f>E42+E43</f>
+        <v/>
+      </c>
+      <c r="F44" s="19">
+        <f>F42+F43</f>
+        <v/>
+      </c>
+      <c r="G44" s="19">
+        <f>G42+G43</f>
+        <v/>
+      </c>
+      <c r="H44" s="19">
+        <f>SUM(B44:G44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>Cash above / (below) reserve</t>
+        </is>
+      </c>
+      <c r="B45" s="19">
+        <f>B44-$B$10</f>
+        <v/>
+      </c>
+      <c r="C45" s="19">
+        <f>C44-$B$10</f>
+        <v/>
+      </c>
+      <c r="D45" s="19">
+        <f>D44-$B$10</f>
+        <v/>
+      </c>
+      <c r="E45" s="19">
+        <f>E44-$B$10</f>
+        <v/>
+      </c>
+      <c r="F45" s="19">
+        <f>F44-$B$10</f>
+        <v/>
+      </c>
+      <c r="G45" s="19">
+        <f>G44-$B$10</f>
+        <v/>
+      </c>
+      <c r="H45" s="19">
+        <f>MIN(B45:G45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>Minimum committed validation capital</t>
+        </is>
+      </c>
+      <c r="B47" s="19">
+        <f>MAX(0,-MIN(B42:G42)+$B$10)</f>
+        <v/>
+      </c>
+      <c r="C47" s="19">
+        <f>B47*10%</f>
+        <v/>
+      </c>
+      <c r="D47" s="19">
+        <f>B47+C47</f>
+        <v/>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>Minimum</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="G47" s="14" t="inlineStr">
+        <is>
+          <t>Recommended total</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFA65E2E"/>
@@ -3912,7 +5072,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF6B5B95"/>
@@ -4232,7 +5392,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="008B5E3C"/>

</xml_diff>